<commit_message>
Add updated Excel files for eb-subc-follow and ipcs, and modify save-as-pdf functionality
</commit_message>
<xml_diff>
--- a/eb-subc-follow.xlsx
+++ b/eb-subc-follow.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d0f35a67bc0854e0/Desktop/ipc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4899" documentId="13_ncr:1_{9E884A3D-A95B-4613-8DC1-BD7A00AA2B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A40CC0E-C294-461B-85E3-60DC3579DE3D}"/>
+  <xr:revisionPtr revIDLastSave="5037" documentId="13_ncr:1_{9E884A3D-A95B-4613-8DC1-BD7A00AA2B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4202E5EC-7A68-4E5C-987B-3E7937EB3161}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="-21504" yWindow="1104" windowWidth="21600" windowHeight="11232" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -145,7 +145,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="350">
   <si>
     <t>#</t>
   </si>
@@ -489,9 +489,6 @@
     <t>Amount log</t>
   </si>
   <si>
-    <t>Chief check</t>
-  </si>
-  <si>
     <t>Discipline signature</t>
   </si>
   <si>
@@ -546,9 +543,6 @@
     <t>Luigong GLG 4215D</t>
   </si>
   <si>
-    <t>Grader</t>
-  </si>
-  <si>
     <t>Printed</t>
   </si>
   <si>
@@ -598,9 +592,6 @@
   </si>
   <si>
     <t>10V288</t>
-  </si>
-  <si>
-    <t>Fuel tanker</t>
   </si>
   <si>
     <t>Quality test</t>
@@ -1101,9 +1092,6 @@
     <t>77VS178</t>
   </si>
   <si>
-    <t>Crane</t>
-  </si>
-  <si>
     <t>77MD834</t>
   </si>
   <si>
@@ -1165,6 +1153,51 @@
   </si>
   <si>
     <t>+994555155362</t>
+  </si>
+  <si>
+    <t>Foldering</t>
+  </si>
+  <si>
+    <t>Mercedes-Benz Actros 3341 Putzmeister 38</t>
+  </si>
+  <si>
+    <t>Kamaz 53-12 Ş-DƏ ATS-3613</t>
+  </si>
+  <si>
+    <t>KAMAZ 5410</t>
+  </si>
+  <si>
+    <t>Dartıcı</t>
+  </si>
+  <si>
+    <t>Su tankeri</t>
+  </si>
+  <si>
+    <t>Ekskavator</t>
+  </si>
+  <si>
+    <t>MERCEDES BENZ YÜK Hi-up</t>
+  </si>
+  <si>
+    <t>Kran</t>
+  </si>
+  <si>
+    <t>KAMAZ 55111</t>
+  </si>
+  <si>
+    <t>KAMAZ</t>
+  </si>
+  <si>
+    <t>ISUZU NPR66</t>
+  </si>
+  <si>
+    <t>Qreyder</t>
+  </si>
+  <si>
+    <t>Beton nasosu</t>
+  </si>
+  <si>
+    <t>Mobil beton nasosu</t>
   </si>
 </sst>
 </file>
@@ -1738,7 +1771,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1956,6 +1989,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" textRotation="180"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2031,8 +2076,8 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -3812,6 +3857,10 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4138,7 +4187,7 @@
   <wetp:taskpane dockstate="right" visibility="0" width="350" row="5">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
-  <wetp:taskpane dockstate="right" visibility="1" width="350" row="5">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="5">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -4194,7 +4243,7 @@
     <col min="6" max="6" width="29.85546875" customWidth="1"/>
     <col min="7" max="7" width="15.140625" style="5" customWidth="1"/>
     <col min="8" max="8" width="3" customWidth="1"/>
-    <col min="9" max="9" width="4.42578125" style="8" customWidth="1"/>
+    <col min="9" max="9" width="4.42578125" style="82" customWidth="1"/>
     <col min="10" max="10" width="6.140625" customWidth="1" outlineLevel="1"/>
     <col min="11" max="13" width="8.28515625" customWidth="1" outlineLevel="2"/>
     <col min="14" max="14" width="18.28515625" customWidth="1" outlineLevel="2"/>
@@ -4203,14 +4252,14 @@
     <col min="17" max="17" width="15.7109375" customWidth="1" outlineLevel="2"/>
     <col min="18" max="18" width="28.140625" customWidth="1" outlineLevel="2"/>
     <col min="19" max="19" width="4" customWidth="1"/>
-    <col min="20" max="20" width="6.7109375" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="21" max="21" width="9" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="22" max="22" width="10" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="23" max="23" width="11.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="24" max="24" width="10.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="25" max="25" width="10.7109375" style="65" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="26" max="26" width="3.5703125" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="27" max="27" width="15.7109375" customWidth="1" collapsed="1"/>
+    <col min="20" max="20" width="6.7109375" customWidth="1" outlineLevel="1"/>
+    <col min="21" max="21" width="9" customWidth="1" outlineLevel="1"/>
+    <col min="22" max="22" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="23" max="23" width="11.28515625" customWidth="1" outlineLevel="1"/>
+    <col min="24" max="24" width="10.28515625" customWidth="1" outlineLevel="1"/>
+    <col min="25" max="25" width="10.7109375" style="65" customWidth="1" outlineLevel="1"/>
+    <col min="26" max="26" width="3.5703125" customWidth="1" outlineLevel="1"/>
+    <col min="27" max="27" width="15.7109375" customWidth="1"/>
     <col min="28" max="28" width="9.85546875" customWidth="1"/>
     <col min="29" max="29" width="8.7109375" customWidth="1"/>
     <col min="30" max="43" width="5.28515625" customWidth="1"/>
@@ -4224,7 +4273,7 @@
         <v>51</v>
       </c>
       <c r="C1" s="76" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D1" s="75" t="s">
         <v>94</v>
@@ -4235,14 +4284,14 @@
       <c r="F1" s="75" t="s">
         <v>50</v>
       </c>
-      <c r="G1" s="75" t="s">
-        <v>336</v>
+      <c r="G1" s="80" t="s">
+        <v>332</v>
       </c>
       <c r="H1" s="75" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="I1" s="75" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="J1" s="7" t="s">
         <v>111</v>
@@ -4251,19 +4300,19 @@
         <v>107</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="M1" s="71" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="N1" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="O1" s="9" t="s">
-        <v>129</v>
+        <v>142</v>
+      </c>
+      <c r="O1" s="108" t="s">
+        <v>128</v>
       </c>
       <c r="P1" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="Q1" s="9" t="s">
         <v>110</v>
@@ -4272,31 +4321,31 @@
         <v>90</v>
       </c>
       <c r="S1" s="77" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="T1" s="57" t="s">
         <v>91</v>
       </c>
       <c r="U1" s="57" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="V1" s="57" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="W1" s="57" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="X1" s="58" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="Y1" s="67" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="Z1" s="57" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="AA1" s="75" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="AB1" s="76" t="s">
         <v>2</v>
@@ -4311,43 +4360,43 @@
         <v>113</v>
       </c>
       <c r="AF1" s="75" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AG1" s="76" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AH1" s="76" t="s">
+        <v>132</v>
+      </c>
+      <c r="AI1" s="76" t="s">
         <v>114</v>
       </c>
-      <c r="AI1" s="76" t="s">
-        <v>134</v>
-      </c>
       <c r="AJ1" s="76" t="s">
-        <v>115</v>
+        <v>133</v>
       </c>
       <c r="AK1" s="76" t="s">
         <v>135</v>
       </c>
       <c r="AL1" s="76" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="AM1" s="76" t="s">
+        <v>140</v>
+      </c>
+      <c r="AN1" s="76" t="s">
+        <v>134</v>
+      </c>
+      <c r="AO1" s="76" t="s">
+        <v>333</v>
+      </c>
+      <c r="AP1" s="76" t="s">
         <v>141</v>
       </c>
-      <c r="AN1" s="76" t="s">
-        <v>142</v>
-      </c>
-      <c r="AO1" s="76" t="s">
-        <v>136</v>
-      </c>
-      <c r="AP1" s="76" t="s">
-        <v>337</v>
-      </c>
       <c r="AQ1" s="76" t="s">
-        <v>143</v>
+        <v>335</v>
       </c>
     </row>
-    <row r="2" spans="1:48">
+    <row r="2" spans="1:48" hidden="1">
       <c r="A2">
         <v>1</v>
       </c>
@@ -4370,13 +4419,13 @@
         <v>30</v>
       </c>
       <c r="G2" s="72" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="H2" s="59" t="str" cm="1">
         <f t="array" ref="H2:H55">IF(_xlfn.DROP(_xlfn._TRO_TRAILING(G:G),1)="","",HYPERLINK("tel://"&amp;MID(_xlfn.DROP(_xlfn._TRO_TRAILING(G:G),1),2,100),"📞"))</f>
         <v>📞</v>
       </c>
-      <c r="I2" s="104" t="str" cm="1">
+      <c r="I2" s="79" t="str" cm="1">
         <f t="array" ref="I2:I55">IF(_xlfn.DROP(_xlfn._TRO_TRAILING(G:G),1)="","",HYPERLINK("https://api.whatsapp.com/send?phone="&amp;MID(_xlfn.DROP(_xlfn._TRO_TRAILING(G:G),1),2,100)&amp;"&amp;text=-","💬"))</f>
         <v>💬</v>
       </c>
@@ -4387,12 +4436,11 @@
         <v>108</v>
       </c>
       <c r="M2" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="N2" s="5"/>
-      <c r="O2" s="5"/>
       <c r="Q2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="R2" t="s">
         <v>67</v>
@@ -4422,26 +4470,32 @@
         <v>14</v>
       </c>
       <c r="AA2" s="10" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="AB2" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC2" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD2" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE2" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF2" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AG2" s="1"/>
-      <c r="AH2" s="1"/>
-      <c r="AI2" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AG2" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AH2" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AI2" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AJ2" s="1"/>
       <c r="AK2" s="1"/>
       <c r="AL2" s="1"/>
@@ -4456,7 +4510,7 @@
       <c r="AU2" s="1"/>
       <c r="AV2" s="1"/>
     </row>
-    <row r="3" spans="1:48">
+    <row r="3" spans="1:48" hidden="1">
       <c r="A3">
         <v>2</v>
       </c>
@@ -4479,12 +4533,12 @@
         <v>31</v>
       </c>
       <c r="G3" s="73" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="H3" s="59" t="str">
         <v>📞</v>
       </c>
-      <c r="I3" s="104" t="str">
+      <c r="I3" s="79" t="str">
         <v>💬</v>
       </c>
       <c r="J3" s="1" t="s">
@@ -4494,12 +4548,11 @@
         <v>108</v>
       </c>
       <c r="M3" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
       <c r="Q3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="R3" t="s">
         <v>66</v>
@@ -4528,23 +4581,29 @@
         <v>11</v>
       </c>
       <c r="AB3" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC3" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD3" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE3" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF3" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AG3" s="1"/>
-      <c r="AH3" s="1"/>
-      <c r="AI3" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AG3" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AH3" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AI3" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AJ3" s="1"/>
       <c r="AK3" s="1"/>
       <c r="AL3" s="1"/>
@@ -4581,8 +4640,8 @@
       <c r="F4" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="60" t="s">
-        <v>235</v>
+      <c r="G4" s="81" t="s">
+        <v>232</v>
       </c>
       <c r="H4" s="59" t="str">
         <v/>
@@ -4601,14 +4660,13 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="N4" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="O4" s="5"/>
       <c r="Q4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="R4" t="s">
         <v>89</v>
@@ -4637,16 +4695,16 @@
         <v>14</v>
       </c>
       <c r="AB4" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC4" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD4" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE4" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF4" s="1"/>
       <c r="AG4" s="1"/>
@@ -4689,7 +4747,7 @@
         <v>28</v>
       </c>
       <c r="G5" s="60" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="H5" s="59" t="str">
         <v/>
@@ -4709,7 +4767,7 @@
       </c>
       <c r="O5" s="5"/>
       <c r="Q5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="R5" t="s">
         <v>89</v>
@@ -4726,12 +4784,8 @@
         <v>14</v>
       </c>
       <c r="Z5" s="2"/>
-      <c r="AB5" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AC5" s="1" t="s">
-        <v>272</v>
-      </c>
+      <c r="AB5" s="1"/>
+      <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
       <c r="AE5" s="1"/>
       <c r="AF5" s="1"/>
@@ -4774,8 +4828,8 @@
       <c r="F6" t="s">
         <v>28</v>
       </c>
-      <c r="G6" s="60" t="s">
-        <v>235</v>
+      <c r="G6" s="81" t="s">
+        <v>232</v>
       </c>
       <c r="H6" s="59" t="str">
         <v/>
@@ -4794,12 +4848,11 @@
         <v/>
       </c>
       <c r="M6" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
       <c r="Q6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="R6" t="s">
         <v>88</v>
@@ -4849,7 +4902,7 @@
       <c r="AU6" s="1"/>
       <c r="AV6" s="1"/>
     </row>
-    <row r="7" spans="1:48" hidden="1">
+    <row r="7" spans="1:48">
       <c r="A7">
         <v>5</v>
       </c>
@@ -4871,8 +4924,8 @@
       <c r="F7" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="60" t="s">
-        <v>235</v>
+      <c r="G7" s="81" t="s">
+        <v>232</v>
       </c>
       <c r="H7" s="59" t="str">
         <v/>
@@ -4891,16 +4944,19 @@
         <v>2</v>
       </c>
       <c r="M7" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="N7" s="70" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="O7" s="62" t="s">
-        <v>317</v>
+        <v>328</v>
+      </c>
+      <c r="P7" t="s">
+        <v>346</v>
       </c>
       <c r="Q7" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="R7" t="s">
         <v>88</v>
@@ -4929,16 +4985,16 @@
         <v>13</v>
       </c>
       <c r="AB7" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC7" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD7" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE7" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF7" s="1"/>
       <c r="AG7" s="1"/>
@@ -4980,8 +5036,8 @@
       <c r="F8" t="s">
         <v>29</v>
       </c>
-      <c r="G8" s="61" t="s">
-        <v>247</v>
+      <c r="G8" s="73" t="s">
+        <v>244</v>
       </c>
       <c r="H8" s="59" t="str">
         <v>📞</v>
@@ -5000,12 +5056,11 @@
         <v/>
       </c>
       <c r="M8" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="N8" s="5"/>
-      <c r="O8" s="5"/>
       <c r="Q8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="R8" t="s">
         <v>87</v>
@@ -5034,16 +5089,16 @@
         <v>18</v>
       </c>
       <c r="AB8" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC8" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD8" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF8" s="1"/>
       <c r="AG8" s="1"/>
@@ -5063,7 +5118,7 @@
       <c r="AU8" s="1"/>
       <c r="AV8" s="1"/>
     </row>
-    <row r="9" spans="1:48" hidden="1">
+    <row r="9" spans="1:48">
       <c r="A9">
         <v>7</v>
       </c>
@@ -5083,10 +5138,10 @@
         <v>46</v>
       </c>
       <c r="F9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G9" s="61" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="H9" s="59" t="str">
         <v>📞</v>
@@ -5105,13 +5160,13 @@
         <v>56</v>
       </c>
       <c r="O9" s="62" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="P9" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="Q9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R9" t="s">
         <v>86</v>
@@ -5161,7 +5216,7 @@
       <c r="AU9" s="1"/>
       <c r="AV9" s="1"/>
     </row>
-    <row r="10" spans="1:48" hidden="1">
+    <row r="10" spans="1:48">
       <c r="A10">
         <v>8</v>
       </c>
@@ -5181,10 +5236,10 @@
         <v>46</v>
       </c>
       <c r="F10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G10" s="61" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H10" s="59" t="str">
         <v>📞</v>
@@ -5203,10 +5258,10 @@
         <v>58</v>
       </c>
       <c r="O10" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="Q10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R10" t="s">
         <v>86</v>
@@ -5245,7 +5300,7 @@
       <c r="AU10" s="1"/>
       <c r="AV10" s="1"/>
     </row>
-    <row r="11" spans="1:48" hidden="1">
+    <row r="11" spans="1:48">
       <c r="A11">
         <v>9</v>
       </c>
@@ -5265,10 +5320,10 @@
         <v>46</v>
       </c>
       <c r="F11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G11" s="61" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H11" s="59" t="str">
         <v>📞</v>
@@ -5287,10 +5342,10 @@
         <v>53</v>
       </c>
       <c r="O11" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="Q11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R11" t="s">
         <v>86</v>
@@ -5329,7 +5384,7 @@
       <c r="AU11" s="1"/>
       <c r="AV11" s="1"/>
     </row>
-    <row r="12" spans="1:48" hidden="1">
+    <row r="12" spans="1:48">
       <c r="A12">
         <v>10</v>
       </c>
@@ -5349,10 +5404,10 @@
         <v>46</v>
       </c>
       <c r="F12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G12" s="61" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H12" s="59" t="str">
         <v>📞</v>
@@ -5371,10 +5426,10 @@
         <v>55</v>
       </c>
       <c r="O12" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="Q12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R12" t="s">
         <v>86</v>
@@ -5413,7 +5468,7 @@
       <c r="AU12" s="1"/>
       <c r="AV12" s="1"/>
     </row>
-    <row r="13" spans="1:48" hidden="1">
+    <row r="13" spans="1:48">
       <c r="A13">
         <v>11</v>
       </c>
@@ -5433,10 +5488,10 @@
         <v>46</v>
       </c>
       <c r="F13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G13" s="61" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H13" s="59" t="str">
         <v>📞</v>
@@ -5455,13 +5510,13 @@
         <v>54</v>
       </c>
       <c r="O13" s="62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P13" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="Q13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R13" t="s">
         <v>86</v>
@@ -5500,7 +5555,7 @@
       <c r="AU13" s="1"/>
       <c r="AV13" s="1"/>
     </row>
-    <row r="14" spans="1:48" hidden="1">
+    <row r="14" spans="1:48">
       <c r="A14">
         <v>12</v>
       </c>
@@ -5520,10 +5575,10 @@
         <v>46</v>
       </c>
       <c r="F14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G14" s="61" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H14" s="59" t="str">
         <v>📞</v>
@@ -5542,10 +5597,10 @@
         <v>57</v>
       </c>
       <c r="O14" s="5" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="Q14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R14" t="s">
         <v>86</v>
@@ -5584,7 +5639,7 @@
       <c r="AU14" s="1"/>
       <c r="AV14" s="1"/>
     </row>
-    <row r="15" spans="1:48" hidden="1">
+    <row r="15" spans="1:48">
       <c r="A15">
         <v>13</v>
       </c>
@@ -5604,10 +5659,10 @@
         <v>46</v>
       </c>
       <c r="F15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G15" s="61" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="H15" s="59" t="str">
         <v>📞</v>
@@ -5626,7 +5681,7 @@
         <v>52</v>
       </c>
       <c r="O15" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="R15" t="s">
         <v>86</v>
@@ -5665,7 +5720,7 @@
       <c r="AU15" s="1"/>
       <c r="AV15" s="1"/>
     </row>
-    <row r="16" spans="1:48" hidden="1">
+    <row r="16" spans="1:48">
       <c r="A16">
         <v>14</v>
       </c>
@@ -5688,7 +5743,7 @@
         <v>32</v>
       </c>
       <c r="G16" s="73" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H16" s="59" t="str">
         <v>📞</v>
@@ -5707,19 +5762,19 @@
         <v>3</v>
       </c>
       <c r="M16" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="N16" s="5" t="s">
         <v>95</v>
       </c>
       <c r="O16" s="62" t="s">
-        <v>133</v>
+        <v>347</v>
       </c>
       <c r="P16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="Q16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R16" t="s">
         <v>85</v>
@@ -5748,24 +5803,26 @@
         <v>9</v>
       </c>
       <c r="AB16" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC16" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD16" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE16" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF16" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AG16" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AH16" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AH16" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AI16" s="1"/>
       <c r="AJ16" s="1"/>
       <c r="AK16" s="1"/>
@@ -5804,12 +5861,12 @@
         <v>33</v>
       </c>
       <c r="G17" s="73" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="H17" s="59" t="str">
         <v>📞</v>
       </c>
-      <c r="I17" s="104" t="str">
+      <c r="I17" s="79" t="str">
         <v>💬</v>
       </c>
       <c r="J17" s="1" t="s">
@@ -5823,19 +5880,19 @@
         <v>4</v>
       </c>
       <c r="M17" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="N17" s="70" t="s">
-        <v>274</v>
-      </c>
-      <c r="O17" s="5" t="s">
-        <v>232</v>
+        <v>271</v>
+      </c>
+      <c r="O17" s="62" t="s">
+        <v>229</v>
       </c>
       <c r="P17" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="Q17" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="R17" t="s">
         <v>84</v>
@@ -5864,19 +5921,19 @@
         <v>7</v>
       </c>
       <c r="AB17" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC17" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD17" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE17" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF17" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AG17" s="1"/>
       <c r="AH17" s="1"/>
@@ -5895,7 +5952,7 @@
       <c r="AU17" s="1"/>
       <c r="AV17" s="1"/>
     </row>
-    <row r="18" spans="1:48" hidden="1">
+    <row r="18" spans="1:48">
       <c r="A18">
         <v>16</v>
       </c>
@@ -5918,7 +5975,7 @@
         <v>33</v>
       </c>
       <c r="G18" s="61" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="H18" s="59" t="str">
         <v>📞</v>
@@ -5937,13 +5994,13 @@
         <v>97</v>
       </c>
       <c r="O18" s="5" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="P18" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="Q18" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="R18" t="s">
         <v>84</v>
@@ -6004,7 +6061,7 @@
         <v>33</v>
       </c>
       <c r="G19" s="61" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="H19" s="59" t="str">
         <v>📞</v>
@@ -6059,7 +6116,7 @@
       <c r="AU19" s="1"/>
       <c r="AV19" s="1"/>
     </row>
-    <row r="20" spans="1:48" hidden="1">
+    <row r="20" spans="1:48">
       <c r="A20">
         <v>18</v>
       </c>
@@ -6082,7 +6139,7 @@
         <v>33</v>
       </c>
       <c r="G20" s="61" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="H20" s="59" t="str">
         <v>📞</v>
@@ -6094,16 +6151,16 @@
         <v>109</v>
       </c>
       <c r="N20" s="5" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="O20" s="62" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="P20" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="Q20" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R20" t="s">
         <v>84</v>
@@ -6141,7 +6198,7 @@
       <c r="AU20" s="1"/>
       <c r="AV20" s="1"/>
     </row>
-    <row r="21" spans="1:48" hidden="1">
+    <row r="21" spans="1:48">
       <c r="A21">
         <v>19</v>
       </c>
@@ -6163,8 +6220,8 @@
       <c r="F21" t="s">
         <v>33</v>
       </c>
-      <c r="G21" s="61" t="s">
-        <v>250</v>
+      <c r="G21" s="73" t="s">
+        <v>247</v>
       </c>
       <c r="H21" s="59" t="str">
         <v>📞</v>
@@ -6183,19 +6240,19 @@
         <v>5</v>
       </c>
       <c r="M21" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="N21" s="70" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="O21" s="62" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="P21" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="Q21" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="R21" t="s">
         <v>84</v>
@@ -6204,26 +6261,24 @@
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
       <c r="W21" s="2"/>
-      <c r="X21">
-        <f t="shared" si="3"/>
-        <v>7</v>
-      </c>
       <c r="Y21" s="65">
         <v>7</v>
       </c>
       <c r="AB21" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC21" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD21" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE21" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AF21" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AF21" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AG21" s="1"/>
       <c r="AH21" s="1"/>
       <c r="AI21" s="1"/>
@@ -6241,7 +6296,7 @@
       <c r="AU21" s="1"/>
       <c r="AV21" s="1"/>
     </row>
-    <row r="22" spans="1:48" hidden="1">
+    <row r="22" spans="1:48">
       <c r="A22">
         <v>20</v>
       </c>
@@ -6263,8 +6318,8 @@
       <c r="F22" t="s">
         <v>33</v>
       </c>
-      <c r="G22" s="61" t="s">
-        <v>250</v>
+      <c r="G22" s="73" t="s">
+        <v>247</v>
       </c>
       <c r="H22" s="59" t="str">
         <v>📞</v>
@@ -6283,19 +6338,19 @@
         <v>6</v>
       </c>
       <c r="M22" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="N22" s="70" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="O22" s="62" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="P22" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="Q22" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="R22" t="s">
         <v>84</v>
@@ -6304,26 +6359,24 @@
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
       <c r="W22" s="2"/>
-      <c r="X22">
-        <f t="shared" si="3"/>
-        <v>7</v>
-      </c>
       <c r="Y22" s="65">
         <v>7</v>
       </c>
       <c r="AB22" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC22" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD22" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE22" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AF22" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AF22" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AG22" s="1"/>
       <c r="AH22" s="1"/>
       <c r="AI22" s="1"/>
@@ -6341,7 +6394,7 @@
       <c r="AU22" s="1"/>
       <c r="AV22" s="1"/>
     </row>
-    <row r="23" spans="1:48" hidden="1">
+    <row r="23" spans="1:48">
       <c r="A23">
         <v>20</v>
       </c>
@@ -6363,8 +6416,8 @@
       <c r="F23" t="s">
         <v>33</v>
       </c>
-      <c r="G23" s="61" t="s">
-        <v>250</v>
+      <c r="G23" s="73" t="s">
+        <v>247</v>
       </c>
       <c r="H23" s="59" t="str">
         <v>📞</v>
@@ -6383,19 +6436,19 @@
         <v>7</v>
       </c>
       <c r="M23" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="N23" s="70" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="O23" s="62" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="P23" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="Q23" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="R23" t="s">
         <v>84</v>
@@ -6404,26 +6457,24 @@
       <c r="U23" s="2"/>
       <c r="V23" s="2"/>
       <c r="W23" s="2"/>
-      <c r="X23">
-        <f t="shared" ref="X23:X24" si="11">IF(Y23="","",Y23)</f>
-        <v>7</v>
-      </c>
       <c r="Y23" s="65">
         <v>7</v>
       </c>
       <c r="AB23" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC23" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD23" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE23" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AF23" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AF23" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AG23" s="1"/>
       <c r="AH23" s="1"/>
       <c r="AI23" s="1"/>
@@ -6501,7 +6552,7 @@
         <v>Open</v>
       </c>
       <c r="X24">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="X24" si="11">IF(Y24="","",Y24)</f>
         <v>4</v>
       </c>
       <c r="Y24" s="65">
@@ -6606,7 +6657,7 @@
       <c r="AU25" s="1"/>
       <c r="AV25" s="1"/>
     </row>
-    <row r="26" spans="1:48" hidden="1">
+    <row r="26" spans="1:48">
       <c r="A26">
         <v>23</v>
       </c>
@@ -6628,8 +6679,8 @@
       <c r="F26" t="s">
         <v>35</v>
       </c>
-      <c r="G26" s="61" t="s">
-        <v>251</v>
+      <c r="G26" s="73" t="s">
+        <v>248</v>
       </c>
       <c r="H26" s="59" t="str">
         <v>📞</v>
@@ -6648,19 +6699,19 @@
         <v>8</v>
       </c>
       <c r="M26" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="N26" s="5" t="s">
         <v>62</v>
       </c>
       <c r="O26" s="62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P26" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="Q26" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R26" t="s">
         <v>82</v>
@@ -6689,24 +6740,26 @@
         <v>10</v>
       </c>
       <c r="AB26" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC26" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD26" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE26" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF26" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AG26" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AH26" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AH26" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AI26" s="1"/>
       <c r="AJ26" s="1"/>
       <c r="AK26" s="1"/>
@@ -6722,7 +6775,7 @@
       <c r="AU26" s="1"/>
       <c r="AV26" s="1"/>
     </row>
-    <row r="27" spans="1:48" hidden="1">
+    <row r="27" spans="1:48">
       <c r="A27">
         <v>24</v>
       </c>
@@ -6745,7 +6798,7 @@
         <v>35</v>
       </c>
       <c r="G27" s="61" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="H27" s="59" t="str">
         <v>📞</v>
@@ -6760,13 +6813,13 @@
         <v>63</v>
       </c>
       <c r="O27" s="62" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P27" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q27" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R27" t="s">
         <v>82</v>
@@ -6828,12 +6881,12 @@
         <v>36</v>
       </c>
       <c r="G28" s="73" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="H28" s="59" t="str">
         <v>📞</v>
       </c>
-      <c r="I28" s="104" t="str">
+      <c r="I28" s="79" t="str">
         <v>💬</v>
       </c>
       <c r="J28" s="1" t="s">
@@ -6847,14 +6900,19 @@
         <v>9</v>
       </c>
       <c r="M28" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="N28" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="O28" s="5"/>
+      <c r="O28" s="62" t="s">
+        <v>349</v>
+      </c>
+      <c r="P28" t="s">
+        <v>336</v>
+      </c>
       <c r="Q28" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="R28" t="s">
         <v>81</v>
@@ -6883,22 +6941,26 @@
         <v>9</v>
       </c>
       <c r="AB28" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC28" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD28" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE28" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF28" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AG28" s="1"/>
-      <c r="AH28" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AG28" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AH28" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AI28" s="1"/>
       <c r="AJ28" s="1"/>
       <c r="AK28" s="1"/>
@@ -6937,12 +6999,12 @@
         <v>37</v>
       </c>
       <c r="G29" s="73" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="H29" s="59" t="str">
         <v>📞</v>
       </c>
-      <c r="I29" s="104" t="str">
+      <c r="I29" s="79" t="str">
         <v>💬</v>
       </c>
       <c r="J29" s="1" t="s">
@@ -6956,16 +7018,19 @@
         <v>10</v>
       </c>
       <c r="M29" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="N29" s="5" t="s">
         <v>101</v>
       </c>
       <c r="O29" s="62" t="s">
-        <v>151</v>
+        <v>340</v>
+      </c>
+      <c r="P29" t="s">
+        <v>337</v>
       </c>
       <c r="Q29" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="R29" t="s">
         <v>80</v>
@@ -6994,22 +7059,26 @@
         <v>8</v>
       </c>
       <c r="AB29" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC29" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD29" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE29" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF29" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AG29" s="1"/>
-      <c r="AH29" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AG29" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AH29" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AI29" s="1"/>
       <c r="AJ29" s="1"/>
       <c r="AK29" s="1"/>
@@ -7048,7 +7117,7 @@
         <v>38</v>
       </c>
       <c r="G30" s="61" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="H30" s="59" t="str">
         <v>📞</v>
@@ -7068,7 +7137,7 @@
       </c>
       <c r="O30" s="5"/>
       <c r="Q30" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="R30" t="s">
         <v>79</v>
@@ -7141,7 +7210,7 @@
         <v>38</v>
       </c>
       <c r="G31" s="61" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="H31" s="59" t="str">
         <v>📞</v>
@@ -7161,7 +7230,7 @@
       </c>
       <c r="O31" s="5"/>
       <c r="Q31" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="R31" t="s">
         <v>79</v>
@@ -7200,7 +7269,7 @@
       <c r="AU31" s="1"/>
       <c r="AV31" s="1"/>
     </row>
-    <row r="32" spans="1:48" hidden="1">
+    <row r="32" spans="1:48">
       <c r="A32">
         <v>29</v>
       </c>
@@ -7222,8 +7291,8 @@
       <c r="F32" t="s">
         <v>39</v>
       </c>
-      <c r="G32" s="61" t="s">
-        <v>254</v>
+      <c r="G32" s="73" t="s">
+        <v>251</v>
       </c>
       <c r="H32" s="59" t="str">
         <v>📞</v>
@@ -7242,19 +7311,19 @@
         <v>11</v>
       </c>
       <c r="M32" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="N32" s="5" t="s">
         <v>102</v>
       </c>
       <c r="O32" s="62" t="s">
-        <v>131</v>
+        <v>341</v>
       </c>
       <c r="P32" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="Q32" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R32" t="s">
         <v>78</v>
@@ -7283,24 +7352,26 @@
         <v>8</v>
       </c>
       <c r="AB32" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC32" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD32" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE32" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF32" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AG32" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AH32" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AH32" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AI32" s="1"/>
       <c r="AJ32" s="1"/>
       <c r="AK32" s="1"/>
@@ -7316,7 +7387,7 @@
       <c r="AU32" s="1"/>
       <c r="AV32" s="1"/>
     </row>
-    <row r="33" spans="1:48" hidden="1">
+    <row r="33" spans="1:48">
       <c r="A33">
         <v>30</v>
       </c>
@@ -7338,8 +7409,8 @@
       <c r="F33" t="s">
         <v>40</v>
       </c>
-      <c r="G33" s="61" t="s">
-        <v>255</v>
+      <c r="G33" s="73" t="s">
+        <v>252</v>
       </c>
       <c r="H33" s="59" t="str">
         <v>📞</v>
@@ -7358,14 +7429,19 @@
         <v>12</v>
       </c>
       <c r="M33" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="N33" s="70" t="s">
         <v>103</v>
       </c>
-      <c r="O33" s="5"/>
+      <c r="O33" s="62" t="s">
+        <v>339</v>
+      </c>
+      <c r="P33" t="s">
+        <v>338</v>
+      </c>
       <c r="Q33" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="R33" t="s">
         <v>77</v>
@@ -7394,28 +7470,32 @@
         <v>8</v>
       </c>
       <c r="AA33" s="10" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="AB33" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC33" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD33" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE33" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF33" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AG33" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AH33" s="1"/>
-      <c r="AI33" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AH33" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AI33" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AJ33" s="1"/>
       <c r="AK33" s="1"/>
       <c r="AL33" s="1"/>
@@ -7453,7 +7533,7 @@
         <v>41</v>
       </c>
       <c r="G34" s="61" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H34" s="59" t="str">
         <v>📞</v>
@@ -7473,7 +7553,7 @@
       </c>
       <c r="O34" s="5"/>
       <c r="Q34" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="R34" t="s">
         <v>76</v>
@@ -7547,12 +7627,12 @@
         <v>42</v>
       </c>
       <c r="G35" s="73" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="H35" s="59" t="str">
         <v>📞</v>
       </c>
-      <c r="I35" s="104" t="str">
+      <c r="I35" s="79" t="str">
         <v>💬</v>
       </c>
       <c r="J35" s="1" t="s">
@@ -7566,19 +7646,19 @@
         <v>13</v>
       </c>
       <c r="M35" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="N35" s="5" t="s">
         <v>105</v>
       </c>
       <c r="O35" s="62" t="s">
-        <v>131</v>
+        <v>341</v>
       </c>
       <c r="P35" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="Q35" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R35" t="s">
         <v>75</v>
@@ -7607,22 +7687,26 @@
         <v>8</v>
       </c>
       <c r="AB35" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC35" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD35" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE35" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF35" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AG35" s="1"/>
-      <c r="AH35" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AG35" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AH35" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AI35" s="1"/>
       <c r="AJ35" s="1"/>
       <c r="AK35" s="1"/>
@@ -7638,7 +7722,7 @@
       <c r="AU35" s="1"/>
       <c r="AV35" s="1"/>
     </row>
-    <row r="36" spans="1:48" hidden="1">
+    <row r="36" spans="1:48">
       <c r="A36">
         <v>32</v>
       </c>
@@ -7661,7 +7745,7 @@
         <v>42</v>
       </c>
       <c r="G36" s="61" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="H36" s="59" t="str">
         <v>📞</v>
@@ -7677,16 +7761,16 @@
         <v/>
       </c>
       <c r="N36" s="5" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="O36" s="62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P36" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="Q36" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R36" t="s">
         <v>75</v>
@@ -7715,7 +7799,7 @@
         <v>8</v>
       </c>
       <c r="AB36" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC36" s="1"/>
       <c r="AD36" s="1"/>
@@ -7761,12 +7845,12 @@
         <v>43</v>
       </c>
       <c r="G37" s="73" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="H37" s="59" t="str">
         <v>📞</v>
       </c>
-      <c r="I37" s="104" t="str">
+      <c r="I37" s="79" t="str">
         <v>💬</v>
       </c>
       <c r="J37" s="1" t="s">
@@ -7780,14 +7864,19 @@
         <v>14</v>
       </c>
       <c r="M37" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="N37" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="O37" s="5"/>
+      <c r="O37" s="62" t="s">
+        <v>340</v>
+      </c>
+      <c r="P37" t="s">
+        <v>344</v>
+      </c>
       <c r="Q37" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="R37" t="s">
         <v>74</v>
@@ -7817,19 +7906,23 @@
       </c>
       <c r="AB37" s="1"/>
       <c r="AC37" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD37" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE37" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF37" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AG37" s="1"/>
-      <c r="AH37" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AG37" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AH37" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AI37" s="1"/>
       <c r="AJ37" s="1"/>
       <c r="AK37" s="1"/>
@@ -7868,7 +7961,7 @@
         <v>43</v>
       </c>
       <c r="G38" s="61" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="H38" s="59" t="str">
         <v>📞</v>
@@ -7888,7 +7981,7 @@
       </c>
       <c r="O38" s="5"/>
       <c r="Q38" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="R38" t="s">
         <v>74</v>
@@ -7927,7 +8020,7 @@
       <c r="AU38" s="1"/>
       <c r="AV38" s="1"/>
     </row>
-    <row r="39" spans="1:48" hidden="1">
+    <row r="39" spans="1:48">
       <c r="A39">
         <v>35</v>
       </c>
@@ -7949,8 +8042,8 @@
       <c r="F39" t="s">
         <v>43</v>
       </c>
-      <c r="G39" s="61" t="s">
-        <v>240</v>
+      <c r="G39" s="73" t="s">
+        <v>237</v>
       </c>
       <c r="H39" s="59" t="str">
         <v>📞</v>
@@ -7969,14 +8062,19 @@
         <v>15</v>
       </c>
       <c r="M39" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="N39" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="O39" s="5"/>
+      <c r="O39" s="62" t="s">
+        <v>340</v>
+      </c>
+      <c r="P39" t="s">
+        <v>345</v>
+      </c>
       <c r="Q39" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="R39" t="s">
         <v>74</v>
@@ -7989,18 +8087,20 @@
         <v>7</v>
       </c>
       <c r="AB39" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC39" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD39" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE39" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AF39" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AF39" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AG39" s="1"/>
       <c r="AH39" s="1"/>
       <c r="AI39" s="1"/>
@@ -8018,7 +8118,7 @@
       <c r="AU39" s="1"/>
       <c r="AV39" s="1"/>
     </row>
-    <row r="40" spans="1:48" hidden="1">
+    <row r="40" spans="1:48">
       <c r="A40">
         <v>36</v>
       </c>
@@ -8040,8 +8140,8 @@
       <c r="F40" t="s">
         <v>43</v>
       </c>
-      <c r="G40" s="60" t="s">
-        <v>236</v>
+      <c r="G40" s="81" t="s">
+        <v>233</v>
       </c>
       <c r="H40" s="59" t="str">
         <v>📞</v>
@@ -8060,14 +8160,19 @@
         <v>16</v>
       </c>
       <c r="M40" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="N40" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="O40" s="5"/>
+      <c r="O40" s="62" t="s">
+        <v>340</v>
+      </c>
+      <c r="P40" t="s">
+        <v>345</v>
+      </c>
       <c r="Q40" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="R40" t="s">
         <v>74</v>
@@ -8076,26 +8181,24 @@
       <c r="U40" s="2"/>
       <c r="V40" s="2"/>
       <c r="W40" s="2"/>
-      <c r="X40">
-        <f t="shared" si="3"/>
-        <v>7</v>
-      </c>
       <c r="Y40" s="65">
         <v>7</v>
       </c>
       <c r="AB40" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC40" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD40" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE40" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AF40" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AF40" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AG40" s="1"/>
       <c r="AH40" s="1"/>
       <c r="AI40" s="1"/>
@@ -8199,7 +8302,7 @@
       <c r="AU41" s="1"/>
       <c r="AV41" s="1"/>
     </row>
-    <row r="42" spans="1:48" hidden="1">
+    <row r="42" spans="1:48">
       <c r="A42">
         <v>38</v>
       </c>
@@ -8222,7 +8325,7 @@
         <v>49</v>
       </c>
       <c r="G42" s="61" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="H42" s="59" t="str">
         <v>📞</v>
@@ -8239,10 +8342,10 @@
       </c>
       <c r="N42" s="5"/>
       <c r="O42" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="Q42" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="R42" t="s">
         <v>72</v>
@@ -8292,7 +8395,7 @@
       <c r="AU42" s="1"/>
       <c r="AV42" s="1"/>
     </row>
-    <row r="43" spans="1:48" hidden="1">
+    <row r="43" spans="1:48">
       <c r="A43">
         <v>39</v>
       </c>
@@ -8314,8 +8417,8 @@
       <c r="F43" t="s">
         <v>44</v>
       </c>
-      <c r="G43" s="61" t="s">
-        <v>258</v>
+      <c r="G43" s="73" t="s">
+        <v>255</v>
       </c>
       <c r="H43" s="59" t="str">
         <v>📞</v>
@@ -8334,14 +8437,19 @@
         <v>17</v>
       </c>
       <c r="M43" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="N43" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="O43" s="5"/>
+      <c r="O43" s="62" t="s">
+        <v>343</v>
+      </c>
+      <c r="P43" t="s">
+        <v>342</v>
+      </c>
       <c r="Q43" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="R43" t="s">
         <v>71</v>
@@ -8369,27 +8477,29 @@
         <v>7</v>
       </c>
       <c r="AA43" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="AB43" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC43" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD43" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE43" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF43" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AG43" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AH43" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AH43" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AI43" s="1"/>
       <c r="AJ43" s="1"/>
       <c r="AK43" s="1"/>
@@ -8491,7 +8601,7 @@
       <c r="AU44" s="1"/>
       <c r="AV44" s="1"/>
     </row>
-    <row r="45" spans="1:48" hidden="1">
+    <row r="45" spans="1:48">
       <c r="A45">
         <v>41</v>
       </c>
@@ -8513,8 +8623,8 @@
       <c r="F45" t="s">
         <v>46</v>
       </c>
-      <c r="G45" s="61" t="s">
-        <v>259</v>
+      <c r="G45" s="73" t="s">
+        <v>256</v>
       </c>
       <c r="H45" s="59" t="str">
         <v>📞</v>
@@ -8533,14 +8643,19 @@
         <v>18</v>
       </c>
       <c r="M45" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="N45" s="70" t="s">
-        <v>122</v>
-      </c>
-      <c r="O45" s="5"/>
+        <v>121</v>
+      </c>
+      <c r="O45" s="62" t="s">
+        <v>339</v>
+      </c>
+      <c r="P45" t="s">
+        <v>338</v>
+      </c>
       <c r="Q45" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="R45" t="s">
         <v>69</v>
@@ -8569,25 +8684,29 @@
         <v>5</v>
       </c>
       <c r="AB45" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC45" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD45" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE45" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF45" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AG45" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AH45" s="1"/>
-      <c r="AI45" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AH45" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AI45" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AJ45" s="1"/>
       <c r="AK45" s="1"/>
       <c r="AL45" s="1"/>
@@ -8701,22 +8820,22 @@
         <v>25</v>
       </c>
       <c r="D47" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E47">
         <f t="shared" si="22"/>
         <v>141</v>
       </c>
       <c r="F47" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="G47" s="73" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="H47" s="59" t="str">
         <v>📞</v>
       </c>
-      <c r="I47" s="104" t="str">
+      <c r="I47" s="79" t="str">
         <v>💬</v>
       </c>
       <c r="J47" s="1" t="s">
@@ -8730,22 +8849,22 @@
         <v>19</v>
       </c>
       <c r="M47" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="N47" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="O47" s="62" t="s">
         <v>150</v>
       </c>
-      <c r="O47" s="62" t="s">
-        <v>153</v>
-      </c>
       <c r="P47" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="Q47" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R47" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="T47" s="2" t="str">
         <f t="shared" si="18"/>
@@ -8771,22 +8890,26 @@
         <v>4</v>
       </c>
       <c r="AB47" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC47" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD47" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE47" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF47" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AG47" s="1"/>
-      <c r="AH47" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AG47" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AH47" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AI47" s="1"/>
       <c r="AJ47" s="1"/>
       <c r="AK47" s="1"/>
@@ -8815,17 +8938,17 @@
         <v>26</v>
       </c>
       <c r="D48" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E48">
         <f t="shared" ref="E48" si="23">_xlfn.NUMBERVALUE(RIGHT(D48,3))</f>
         <v>150</v>
       </c>
       <c r="F48" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="G48" s="61" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="H48" s="59" t="str">
         <v>📞</v>
@@ -8843,10 +8966,10 @@
       <c r="N48" s="5"/>
       <c r="O48" s="4"/>
       <c r="Q48" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="R48" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="T48" s="2" t="str">
         <f t="shared" si="18"/>
@@ -8872,7 +8995,7 @@
         <v>1</v>
       </c>
       <c r="AA48" s="10" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="AB48" s="1"/>
       <c r="AC48" s="1"/>
@@ -8896,7 +9019,7 @@
       <c r="AU48" s="1"/>
       <c r="AV48" s="1"/>
     </row>
-    <row r="49" spans="1:48" hidden="1">
+    <row r="49" spans="1:48">
       <c r="A49">
         <v>45</v>
       </c>
@@ -8909,10 +9032,10 @@
         <v>27</v>
       </c>
       <c r="D49" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="F49" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="G49"/>
       <c r="H49" s="59" t="str">
@@ -8922,26 +9045,26 @@
         <v/>
       </c>
       <c r="J49" s="1" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="L49" t="str">
         <f>IF(OR(K49="",N49=""),"",MAX(L$2:L48)+1)</f>
         <v/>
       </c>
       <c r="N49" s="5" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="O49" s="62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P49" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="Q49" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R49" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="T49" s="2" t="str">
         <f t="shared" ref="T49" si="24">HYPERLINK(subc_contr_folder_path&amp;R49,"Open")</f>
@@ -9001,17 +9124,17 @@
         <v>28</v>
       </c>
       <c r="D50" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="E50">
         <f t="shared" ref="E50:E54" si="26">_xlfn.NUMBERVALUE(RIGHT(D50,3))</f>
         <v>163</v>
       </c>
       <c r="F50" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="G50" s="74" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="H50" t="str">
         <v>📞</v>
@@ -9030,22 +9153,22 @@
         <v>20</v>
       </c>
       <c r="M50" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
       <c r="N50" s="5" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="O50" s="62" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="P50" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="Q50" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="R50" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="T50" s="2" t="str">
         <f t="shared" ref="T50" si="27">HYPERLINK(subc_contr_folder_path&amp;R50,"Open")</f>
@@ -9072,19 +9195,23 @@
       </c>
       <c r="AB50" s="1"/>
       <c r="AC50" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD50" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE50" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF50" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AG50" s="1"/>
-      <c r="AH50" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AG50" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AH50" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AI50" s="1"/>
       <c r="AJ50" s="1"/>
       <c r="AK50" s="1"/>
@@ -9100,7 +9227,7 @@
       <c r="AU50" s="1"/>
       <c r="AV50" s="1"/>
     </row>
-    <row r="51" spans="1:48" hidden="1">
+    <row r="51" spans="1:48">
       <c r="A51">
         <v>48</v>
       </c>
@@ -9113,17 +9240,17 @@
         <v>29</v>
       </c>
       <c r="D51" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="E51">
         <f t="shared" si="26"/>
         <v>164</v>
       </c>
       <c r="F51" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G51" s="63" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="H51" t="str">
         <v>📞</v>
@@ -9139,19 +9266,19 @@
         <v/>
       </c>
       <c r="N51" s="5" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="O51" s="62" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="P51" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="Q51" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="R51" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="T51" s="2" t="str">
         <f t="shared" ref="T51" si="28">HYPERLINK(subc_contr_folder_path&amp;R51,"Open")</f>
@@ -9211,22 +9338,22 @@
         <v>30</v>
       </c>
       <c r="D52" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="E52">
         <f t="shared" si="26"/>
         <v>172</v>
       </c>
       <c r="F52" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="G52" s="74" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="H52" t="str">
         <v>📞</v>
       </c>
-      <c r="I52" s="8" t="str">
+      <c r="I52" s="82" t="str">
         <v>💬</v>
       </c>
       <c r="J52" s="1" t="s">
@@ -9240,22 +9367,22 @@
         <v>21</v>
       </c>
       <c r="M52" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="N52" s="5" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="O52" s="62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="P52" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="Q52" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R52" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="T52" s="2" t="str">
         <f t="shared" ref="T52" si="30">HYPERLINK(subc_contr_folder_path&amp;R52,"Open")</f>
@@ -9281,22 +9408,22 @@
         <v>2</v>
       </c>
       <c r="AA52" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="AB52" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC52" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD52" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE52" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF52" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AG52" s="1"/>
       <c r="AH52" s="1"/>
@@ -9328,22 +9455,22 @@
         <v>31</v>
       </c>
       <c r="D53" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E53">
         <f t="shared" si="26"/>
         <v>173</v>
       </c>
       <c r="F53" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="G53" s="74" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="H53" t="str">
         <v>📞</v>
       </c>
-      <c r="I53" s="8" t="str">
+      <c r="I53" s="82" t="str">
         <v>💬</v>
       </c>
       <c r="J53" s="1" t="s">
@@ -9357,22 +9484,22 @@
         <v>22</v>
       </c>
       <c r="M53" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="N53" s="5" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="O53" s="62" t="s">
-        <v>286</v>
+        <v>348</v>
       </c>
       <c r="P53" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="Q53" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="R53" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="T53" s="2" t="str">
         <f t="shared" ref="T53" si="31">HYPERLINK(subc_contr_folder_path&amp;R53,"Open")</f>
@@ -9398,22 +9525,26 @@
         <v>1</v>
       </c>
       <c r="AB53" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC53" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD53" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE53" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AF53" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AG53" s="1"/>
-      <c r="AH53" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AG53" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AH53" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AI53" s="1"/>
       <c r="AJ53" s="1"/>
       <c r="AK53" s="1"/>
@@ -9429,7 +9560,7 @@
       <c r="AU53" s="1"/>
       <c r="AV53" s="1"/>
     </row>
-    <row r="54" spans="1:48" hidden="1">
+    <row r="54" spans="1:48">
       <c r="A54">
         <v>51</v>
       </c>
@@ -9442,22 +9573,22 @@
         <v>32</v>
       </c>
       <c r="D54" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="E54">
         <f t="shared" si="26"/>
         <v>182</v>
       </c>
       <c r="F54" t="s">
-        <v>331</v>
-      </c>
-      <c r="G54" s="63" t="s">
-        <v>315</v>
+        <v>327</v>
+      </c>
+      <c r="G54" s="74" t="s">
+        <v>312</v>
       </c>
       <c r="H54" t="str">
         <v>📞</v>
       </c>
-      <c r="I54" t="str">
+      <c r="I54" s="4" t="str">
         <v>💬</v>
       </c>
       <c r="J54" s="1" t="s">
@@ -9471,41 +9602,67 @@
         <v>23</v>
       </c>
       <c r="M54" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="N54" s="70" t="s">
-        <v>316</v>
-      </c>
-      <c r="O54" t="s">
-        <v>332</v>
+        <v>313</v>
+      </c>
+      <c r="O54" s="62" t="s">
+        <v>328</v>
       </c>
       <c r="P54" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="Q54" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="R54" t="s">
-        <v>330</v>
+        <v>326</v>
+      </c>
+      <c r="T54" s="2" t="str">
+        <f t="shared" ref="T54" si="33">HYPERLINK(subc_contr_folder_path&amp;R54,"Open")</f>
+        <v>Open</v>
+      </c>
+      <c r="U54" s="2" t="str">
+        <f>HYPERLINK(subc_contr_folder_path&amp;R54&amp;"\ipcs\"&amp;X54,"Open")</f>
+        <v>Open</v>
+      </c>
+      <c r="V54" s="2" t="str">
+        <f t="shared" ref="V54" si="34">HYPERLINK(subc_contr_folder_path&amp;R54&amp;"\ipcs\"&amp;X54&amp;"\"&amp;"log.pdf","Open")</f>
+        <v>Open</v>
+      </c>
+      <c r="W54" s="2" t="str">
+        <f t="shared" ref="W54" si="35">HYPERLINK(subc_contr_folder_path&amp;R54&amp;"\ipcs\"&amp;X54&amp;"\"&amp;E54&amp;"-"&amp;X54&amp;".pdf","Open")</f>
+        <v>Open</v>
+      </c>
+      <c r="X54">
+        <f t="shared" ref="X54" si="36">IF(Y54="","",Y54)</f>
+        <v>1</v>
       </c>
       <c r="Y54" s="65">
         <v>1</v>
       </c>
       <c r="AB54" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC54" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD54" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE54" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AF54" s="1"/>
-      <c r="AG54" s="1"/>
-      <c r="AH54" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AF54" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AG54" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="AH54" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AI54" s="1"/>
       <c r="AJ54" s="1"/>
       <c r="AK54" s="1"/>
@@ -9521,12 +9678,12 @@
       <c r="AU54" s="1"/>
       <c r="AV54" s="1"/>
     </row>
-    <row r="55" spans="1:48" hidden="1">
+    <row r="55" spans="1:48">
       <c r="A55">
         <v>51</v>
       </c>
       <c r="B55">
-        <f t="shared" ref="B55" ca="1" si="33">COUNTIF(INDIRECT("D1:D"&amp;ROW()-1),D55)+1</f>
+        <f t="shared" ref="B55" ca="1" si="37">COUNTIF(INDIRECT("D1:D"&amp;ROW()-1),D55)+1</f>
         <v>2</v>
       </c>
       <c r="C55" t="str">
@@ -9534,17 +9691,17 @@
         <v/>
       </c>
       <c r="D55" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="E55">
-        <f t="shared" ref="E55" si="34">_xlfn.NUMBERVALUE(RIGHT(D55,3))</f>
+        <f t="shared" ref="E55" si="38">_xlfn.NUMBERVALUE(RIGHT(D55,3))</f>
         <v>182</v>
       </c>
       <c r="F55" t="s">
-        <v>331</v>
-      </c>
-      <c r="G55" s="63" t="s">
-        <v>315</v>
+        <v>327</v>
+      </c>
+      <c r="G55" s="74" t="s">
+        <v>312</v>
       </c>
       <c r="H55" t="str">
         <v>📞</v>
@@ -9563,39 +9720,41 @@
         <v>24</v>
       </c>
       <c r="M55" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="N55" s="70" t="s">
-        <v>318</v>
-      </c>
-      <c r="O55" t="s">
-        <v>332</v>
+        <v>314</v>
+      </c>
+      <c r="O55" s="62" t="s">
+        <v>328</v>
       </c>
       <c r="P55" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="Q55" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="R55" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="Y55" s="65">
         <v>1</v>
       </c>
       <c r="AB55" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AC55" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AD55" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="AE55" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="AF55" s="1"/>
+        <v>269</v>
+      </c>
+      <c r="AF55" s="1" t="s">
+        <v>269</v>
+      </c>
       <c r="AG55" s="1"/>
       <c r="AH55" s="1"/>
       <c r="AI55" s="1"/>
@@ -9937,23 +10096,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AQ55" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="10">
+    <filterColumn colId="14">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
-    </filterColumn>
-    <filterColumn colId="19">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-    <filterColumn colId="31">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-    <filterColumn colId="32">
-      <filters blank="1"/>
     </filterColumn>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="R2:R46">
@@ -10378,37 +10524,37 @@
     <row r="1" spans="1:31" ht="25.5" customHeight="1" thickBot="1">
       <c r="A1" s="11"/>
       <c r="B1" s="12"/>
-      <c r="C1" s="86" t="str">
+      <c r="C1" s="90" t="str">
         <f>"KİRALIK ARAÇ GÜNLÜK PUANTAJ TAKİP FORMU - "&amp;RIGHT(I4,3)&amp;" - "&amp;_xlfn.XLOOKUP(I4,data!D:D,data!Y:Y,,0)+M4</f>
         <v>KİRALIK ARAÇ GÜNLÜK PUANTAJ TAKİP FORMU - 163 - 3</v>
       </c>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
-      <c r="H1" s="86"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="83"/>
+      <c r="J1" s="83"/>
     </row>
     <row r="2" spans="1:31" ht="43.5" customHeight="1" thickBot="1">
       <c r="A2" s="13"/>
       <c r="B2" s="13"/>
-      <c r="C2" s="87"/>
-      <c r="D2" s="87"/>
-      <c r="E2" s="87"/>
-      <c r="F2" s="87"/>
-      <c r="G2" s="87"/>
-      <c r="H2" s="87"/>
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
+      <c r="H2" s="91"/>
       <c r="I2" s="13"/>
       <c r="J2" s="13"/>
       <c r="L2" s="44" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="M2" s="45" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="N2" s="45" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="O2" s="45" t="s">
         <v>110</v>
@@ -10418,10 +10564,10 @@
         <v>Department</v>
       </c>
       <c r="U2" s="43" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="V2" s="43" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="W2" s="43"/>
       <c r="X2" s="43"/>
@@ -10434,26 +10580,26 @@
       <c r="AE2" s="43"/>
     </row>
     <row r="3" spans="1:31" ht="26.25" customHeight="1" thickBot="1">
-      <c r="A3" s="88" t="s">
-        <v>178</v>
-      </c>
-      <c r="B3" s="88"/>
-      <c r="C3" s="82" t="str">
+      <c r="A3" s="92" t="s">
+        <v>175</v>
+      </c>
+      <c r="B3" s="92"/>
+      <c r="C3" s="86" t="str">
         <f>_xlfn.XLOOKUP(L3,data!L:L,data!F:F,,0)</f>
         <v>Əsgərov Yaşar</v>
       </c>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83"/>
-      <c r="G3" s="88" t="s">
-        <v>181</v>
-      </c>
-      <c r="H3" s="89"/>
-      <c r="I3" s="80" t="str">
+      <c r="D3" s="87"/>
+      <c r="E3" s="87"/>
+      <c r="F3" s="87"/>
+      <c r="G3" s="92" t="s">
+        <v>178</v>
+      </c>
+      <c r="H3" s="93"/>
+      <c r="I3" s="84" t="str">
         <f>VLOOKUP(M3,Z3:AB14,2,0)&amp;" "&amp;N3</f>
         <v>FEVRAL 2026</v>
       </c>
-      <c r="J3" s="81"/>
+      <c r="J3" s="85"/>
       <c r="L3" s="46">
         <v>20</v>
       </c>
@@ -10471,10 +10617,10 @@
         <v>QA/QC</v>
       </c>
       <c r="U3" s="43" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="V3" s="43" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="W3" s="43"/>
       <c r="X3" s="43"/>
@@ -10487,7 +10633,7 @@
         <v>YANVAR</v>
       </c>
       <c r="AB3" s="43" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="AC3" s="43"/>
       <c r="AD3" s="43"/>
@@ -10495,25 +10641,25 @@
     </row>
     <row r="4" spans="1:31" ht="26.25" customHeight="1" thickBot="1">
       <c r="A4" s="15" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B4" s="14"/>
-      <c r="C4" s="82" t="str" cm="1">
+      <c r="C4" s="86" t="str" cm="1">
         <f t="array" ref="C4">INDEX(_xlfn.TEXTSPLIT(_xlfn.XLOOKUP(L3,data!L:L,data!N:N,,0),"-"),1)</f>
         <v>110FA930</v>
       </c>
-      <c r="D4" s="83"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="83"/>
-      <c r="G4" s="88" t="s">
-        <v>230</v>
-      </c>
-      <c r="H4" s="89"/>
-      <c r="I4" s="98" t="str">
+      <c r="D4" s="87"/>
+      <c r="E4" s="87"/>
+      <c r="F4" s="87"/>
+      <c r="G4" s="92" t="s">
+        <v>227</v>
+      </c>
+      <c r="H4" s="93"/>
+      <c r="I4" s="102" t="str">
         <f>_xlfn.XLOOKUP(L3,data!L:L,data!D:D,,0)</f>
         <v>KLN-SPP2-EQ-163</v>
       </c>
-      <c r="J4" s="81"/>
+      <c r="J4" s="85"/>
       <c r="L4" s="69">
         <v>183</v>
       </c>
@@ -10526,10 +10672,10 @@
         <v>Workshop</v>
       </c>
       <c r="U4" s="43" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="V4" s="43" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="W4" s="43"/>
       <c r="X4" s="43"/>
@@ -10542,7 +10688,7 @@
         <v>FEVRAL</v>
       </c>
       <c r="AB4" s="43" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="AC4" s="43"/>
       <c r="AD4" s="43"/>
@@ -10550,33 +10696,33 @@
     </row>
     <row r="5" spans="1:31" ht="26.25" customHeight="1">
       <c r="A5" s="15" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B5" s="14"/>
-      <c r="C5" s="82" t="str">
+      <c r="C5" s="86" t="str">
         <f>_xlfn.XLOOKUP(L3,data!L:L,data!P:P,,0)</f>
         <v>Komatsu</v>
       </c>
-      <c r="D5" s="83"/>
-      <c r="E5" s="83"/>
-      <c r="F5" s="83"/>
-      <c r="G5" s="88" t="s">
-        <v>271</v>
-      </c>
-      <c r="H5" s="89"/>
-      <c r="I5" s="80">
+      <c r="D5" s="87"/>
+      <c r="E5" s="87"/>
+      <c r="F5" s="87"/>
+      <c r="G5" s="92" t="s">
+        <v>268</v>
+      </c>
+      <c r="H5" s="93"/>
+      <c r="I5" s="84">
         <f>_xlfn.XLOOKUP(I4,data!D:D,data!Y:Y,,0)+M4</f>
         <v>3</v>
       </c>
-      <c r="J5" s="81"/>
+      <c r="J5" s="85"/>
       <c r="T5" s="43" t="str">
         <v>Administration</v>
       </c>
       <c r="U5" s="43" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="V5" s="43" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="W5" s="43"/>
       <c r="X5" s="43"/>
@@ -10589,7 +10735,7 @@
         <v>MART</v>
       </c>
       <c r="AB5" s="43" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="AC5" s="43"/>
       <c r="AD5" s="43"/>
@@ -10597,25 +10743,25 @@
     </row>
     <row r="6" spans="1:31" ht="26.25" customHeight="1" thickBot="1">
       <c r="A6" s="15" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B6" s="14"/>
-      <c r="C6" s="84" t="str">
+      <c r="C6" s="88" t="str">
         <f>IF(RIGHT(_xlfn.XLOOKUP(L3,data!L:L,data!N:N,,0))="N","GECƏ","")</f>
         <v/>
       </c>
-      <c r="D6" s="85"/>
-      <c r="E6" s="85"/>
-      <c r="F6" s="85"/>
-      <c r="G6" s="88" t="s">
-        <v>179</v>
-      </c>
-      <c r="H6" s="89"/>
-      <c r="I6" s="90" t="str">
+      <c r="D6" s="89"/>
+      <c r="E6" s="89"/>
+      <c r="F6" s="89"/>
+      <c r="G6" s="92" t="s">
+        <v>176</v>
+      </c>
+      <c r="H6" s="93"/>
+      <c r="I6" s="94" t="str">
         <f>"+"&amp;MID(_xlfn.XLOOKUP(L3,data!L:L,data!G:G,,0),2,12)</f>
         <v>+994558864957</v>
       </c>
-      <c r="J6" s="91"/>
+      <c r="J6" s="95"/>
       <c r="O6" t="e" cm="1" vm="1">
         <f t="array" ref="O6">_xlfn._xlws.FILTER(_xlfn._TRO_TRAILING(data!L:L),IFERROR(_xlfn.NUMBERVALUE(RIGHT(_xlfn._TRO_TRAILING(data!D:D),3)),"")=L4)</f>
         <v>#VALUE!</v>
@@ -10624,10 +10770,10 @@
         <v>Vinç sepet</v>
       </c>
       <c r="U6" s="43" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="V6" s="43" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="W6" s="43"/>
       <c r="X6" s="43"/>
@@ -10640,7 +10786,7 @@
         <v>APREL</v>
       </c>
       <c r="AB6" s="43" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="AC6" s="43"/>
       <c r="AD6" s="43"/>
@@ -10648,44 +10794,44 @@
     </row>
     <row r="7" spans="1:31" ht="54" customHeight="1" thickBot="1">
       <c r="A7" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="D7" s="17" t="s">
         <v>182</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="E7" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="F7" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="G7" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="H7" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="I7" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="J7" s="19" t="s">
         <v>188</v>
-      </c>
-      <c r="H7" s="18" t="s">
-        <v>189</v>
-      </c>
-      <c r="I7" s="18" t="s">
-        <v>190</v>
-      </c>
-      <c r="J7" s="19" t="s">
-        <v>191</v>
       </c>
       <c r="N7" s="64"/>
       <c r="T7" s="43" t="str">
         <v>Earthworks</v>
       </c>
       <c r="U7" s="43" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="V7" s="43" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="W7" s="43"/>
       <c r="X7" s="43"/>
@@ -10698,7 +10844,7 @@
         <v>MAY</v>
       </c>
       <c r="AB7" s="43" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="AC7" s="43"/>
       <c r="AD7" s="43"/>
@@ -10730,10 +10876,10 @@
         <v>0</v>
       </c>
       <c r="U8" s="43" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="V8" s="43" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="W8" s="43"/>
       <c r="X8" s="43"/>
@@ -10746,7 +10892,7 @@
         <v>IYUN</v>
       </c>
       <c r="AB8" s="43" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="AC8" s="43"/>
       <c r="AD8" s="43"/>
@@ -10774,10 +10920,10 @@
         <v>Rough Works</v>
       </c>
       <c r="U9" s="43" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="V9" s="43" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="W9" s="43"/>
       <c r="X9" s="43"/>
@@ -10790,7 +10936,7 @@
         <v>IYUL</v>
       </c>
       <c r="AB9" s="43" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="AC9" s="43"/>
       <c r="AD9" s="43"/>
@@ -10821,10 +10967,10 @@
         <v>Warehouse</v>
       </c>
       <c r="U10" s="43" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="V10" s="43" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="W10" s="43"/>
       <c r="X10" s="43"/>
@@ -10837,7 +10983,7 @@
         <v>AVQUST</v>
       </c>
       <c r="AB10" s="43" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="AC10" s="43"/>
       <c r="AD10" s="43"/>
@@ -10868,10 +11014,10 @@
         <v>HSE</v>
       </c>
       <c r="U11" s="43" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="V11" s="43" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="W11" s="43"/>
       <c r="X11" s="43"/>
@@ -10884,7 +11030,7 @@
         <v>SENTYABR</v>
       </c>
       <c r="AB11" s="43" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="AC11" s="43"/>
       <c r="AD11" s="43"/>
@@ -10926,7 +11072,7 @@
         <v>OKTYABR</v>
       </c>
       <c r="AB12" s="43" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="AC12" s="43"/>
       <c r="AD12" s="43"/>
@@ -10966,7 +11112,7 @@
         <v>NOYABR</v>
       </c>
       <c r="AB13" s="43" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="AC13" s="43"/>
       <c r="AD13" s="43"/>
@@ -11006,7 +11152,7 @@
         <v>DEKABR</v>
       </c>
       <c r="AB14" s="43" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="AC14" s="43"/>
       <c r="AD14" s="43"/>
@@ -11519,21 +11665,21 @@
     <row r="39" spans="1:12" ht="33.75" customHeight="1" thickBot="1">
       <c r="A39" s="34"/>
       <c r="B39" s="51" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="C39" s="52">
         <f>+COUNTA(C8:C38)</f>
         <v>0</v>
       </c>
       <c r="D39" s="51" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="E39" s="52">
         <f>+COUNTA(E8:E38)</f>
         <v>0</v>
       </c>
       <c r="F39" s="54" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G39" s="56">
         <f>SUM(G8:G38)</f>
@@ -11548,80 +11694,80 @@
     </row>
     <row r="40" spans="1:12" ht="31.5" customHeight="1" thickBot="1">
       <c r="A40" s="41" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B40" s="42"/>
       <c r="C40" s="42"/>
-      <c r="D40" s="101" t="s">
-        <v>217</v>
-      </c>
-      <c r="E40" s="102"/>
-      <c r="F40" s="103"/>
-      <c r="G40" s="95" t="s">
-        <v>192</v>
-      </c>
-      <c r="H40" s="96"/>
-      <c r="I40" s="97"/>
+      <c r="D40" s="105" t="s">
+        <v>214</v>
+      </c>
+      <c r="E40" s="106"/>
+      <c r="F40" s="107"/>
+      <c r="G40" s="99" t="s">
+        <v>189</v>
+      </c>
+      <c r="H40" s="100"/>
+      <c r="I40" s="101"/>
       <c r="J40" s="38" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="31.5" customHeight="1" thickBot="1">
-      <c r="A41" s="99" t="str">
+      <c r="A41" s="103" t="str">
         <f>_xlfn.XLOOKUP(L3,data!L:L,data!F:F)</f>
         <v>Əsgərov Yaşar</v>
       </c>
-      <c r="B41" s="100"/>
-      <c r="C41" s="100"/>
-      <c r="D41" s="92"/>
-      <c r="E41" s="93"/>
-      <c r="F41" s="94"/>
-      <c r="G41" s="95"/>
-      <c r="H41" s="96"/>
-      <c r="I41" s="97"/>
+      <c r="B41" s="104"/>
+      <c r="C41" s="104"/>
+      <c r="D41" s="96"/>
+      <c r="E41" s="97"/>
+      <c r="F41" s="98"/>
+      <c r="G41" s="99"/>
+      <c r="H41" s="100"/>
+      <c r="I41" s="101"/>
       <c r="J41" s="39"/>
     </row>
     <row r="42" spans="1:12" ht="33.6" customHeight="1" thickBot="1">
       <c r="A42" s="41" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B42" s="42"/>
       <c r="C42" s="42"/>
-      <c r="D42" s="92" t="str">
+      <c r="D42" s="96" t="str">
         <f>VLOOKUP(O3,T2:V10,2,0)</f>
         <v>Ambar şefi</v>
       </c>
-      <c r="E42" s="93"/>
-      <c r="F42" s="94"/>
-      <c r="G42" s="95" t="str">
+      <c r="E42" s="97"/>
+      <c r="F42" s="98"/>
+      <c r="G42" s="99" t="str">
         <f>VLOOKUP(O3,T2:V10,3,0)</f>
         <v>Ibrahim Akgün</v>
       </c>
-      <c r="H42" s="96"/>
-      <c r="I42" s="97"/>
+      <c r="H42" s="100"/>
+      <c r="I42" s="101"/>
       <c r="J42" s="40"/>
     </row>
     <row r="43" spans="1:12" ht="33.6" customHeight="1" thickBot="1">
       <c r="A43" s="41" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B43" s="42"/>
       <c r="C43" s="42"/>
-      <c r="D43" s="92" t="s">
-        <v>218</v>
-      </c>
-      <c r="E43" s="93"/>
-      <c r="F43" s="94"/>
-      <c r="G43" s="95" t="s">
-        <v>220</v>
-      </c>
-      <c r="H43" s="96"/>
-      <c r="I43" s="97"/>
+      <c r="D43" s="96" t="s">
+        <v>215</v>
+      </c>
+      <c r="E43" s="97"/>
+      <c r="F43" s="98"/>
+      <c r="G43" s="99" t="s">
+        <v>217</v>
+      </c>
+      <c r="H43" s="100"/>
+      <c r="I43" s="101"/>
       <c r="J43" s="40"/>
     </row>
     <row r="44" spans="1:12" ht="39" customHeight="1">
       <c r="A44" s="48" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B44" s="48"/>
     </row>
@@ -11705,12 +11851,12 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="6" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="B2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -11729,7 +11875,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>65</v>
@@ -11737,35 +11883,35 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="6" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B4" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C4" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B5" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C5" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add new files and update project structure
- Added new Excel files: eb-subc-follow.xlsx, log_daily_records.xlsx, and read_ipc_dates.xlsx.
- Added images: akk.png, akk2.png, and logo.png.
- Updated .gitignore to exclude specific PDF patterns.
- Created main.py and readFiles.py scripts for reading Excel files.
- Added pyproject.toml for project dependencies and metadata.
- Introduced uv.lock for dependency resolution.
- Updated README.md for project documentation.
</commit_message>
<xml_diff>
--- a/eb-subc-follow.xlsx
+++ b/eb-subc-follow.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d0f35a67bc0854e0/Desktop/ipc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6110" documentId="13_ncr:1_{9E884A3D-A95B-4613-8DC1-BD7A00AA2B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E0AB1ED-C41C-490C-9129-83AFA28716B9}"/>
+  <xr:revisionPtr revIDLastSave="6126" documentId="13_ncr:1_{9E884A3D-A95B-4613-8DC1-BD7A00AA2B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79D7D7FF-EB8E-436E-ACF6-84B9E0E4D718}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3855" yWindow="3855" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -79,7 +79,7 @@
     <definedName name="xxxx" localSheetId="1" hidden="1">{#N/A,#N/A,FALSE,"D1";#N/A,#N/A,FALSE,"D2";#N/A,#N/A,FALSE,"D3";#N/A,#N/A,FALSE,"D4";#N/A,#N/A,FALSE,"D5";#N/A,#N/A,FALSE,"D6";#N/A,#N/A,FALSE,"D7";#N/A,#N/A,FALSE,"D8";#N/A,#N/A,FALSE,"D9";#N/A,#N/A,FALSE,"D10";#N/A,#N/A,FALSE,"D11";#N/A,#N/A,FALSE,"D12";#N/A,#N/A,FALSE,"D13";#N/A,#N/A,FALSE,"D14";#N/A,#N/A,FALSE,"D15";#N/A,#N/A,FALSE,"D16"}</definedName>
     <definedName name="xxxx" hidden="1">{#N/A,#N/A,FALSE,"D1";#N/A,#N/A,FALSE,"D2";#N/A,#N/A,FALSE,"D3";#N/A,#N/A,FALSE,"D4";#N/A,#N/A,FALSE,"D5";#N/A,#N/A,FALSE,"D6";#N/A,#N/A,FALSE,"D7";#N/A,#N/A,FALSE,"D8";#N/A,#N/A,FALSE,"D9";#N/A,#N/A,FALSE,"D10";#N/A,#N/A,FALSE,"D11";#N/A,#N/A,FALSE,"D12";#N/A,#N/A,FALSE,"D13";#N/A,#N/A,FALSE,"D14";#N/A,#N/A,FALSE,"D15";#N/A,#N/A,FALSE,"D16"}</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -2451,7 +2451,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="22" fmlaLink="$L$3" max="50" min="1" page="10" val="31"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="22" fmlaLink="$L$3" max="50" min="1" page="10" val="21"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2618,10 +2618,10 @@
       <sheetName val="view__cover"/>
       <sheetName val="view_calc"/>
       <sheetName val="view_daily_records"/>
+      <sheetName val="view_fuel"/>
+      <sheetName val="log_daily_records"/>
+      <sheetName val="log_monthly_records"/>
       <sheetName val="view_monthly_records"/>
-      <sheetName val="view_fuel"/>
-      <sheetName val="log_monthly_records"/>
-      <sheetName val="log_daily_records"/>
       <sheetName val="log_ipcs"/>
       <sheetName val="log_contracts"/>
       <sheetName val="log_addendums"/>
@@ -2633,13 +2633,7 @@
       <sheetName val="old_ipc_dates"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0">
-        <row r="1">
-          <cell r="R1">
-            <v>31</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="0"/>
       <sheetData sheetId="1"/>
       <sheetData sheetId="2"/>
       <sheetData sheetId="3"/>
@@ -2648,1699 +2642,8 @@
       <sheetData sheetId="6"/>
       <sheetData sheetId="7">
         <row r="1">
-          <cell r="C1" t="str">
-            <v>contract no</v>
-          </cell>
-          <cell r="D1" t="str">
-            <v>no</v>
-          </cell>
-        </row>
-        <row r="2">
-          <cell r="C2">
-            <v>30</v>
-          </cell>
-          <cell r="D2">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="3">
-          <cell r="C3">
-            <v>31</v>
-          </cell>
-          <cell r="D3">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="4">
-          <cell r="C4">
-            <v>46</v>
-          </cell>
-          <cell r="D4">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="C5">
-            <v>50</v>
-          </cell>
-          <cell r="D5">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="C6">
-            <v>51</v>
-          </cell>
-          <cell r="D6">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="C7">
-            <v>52</v>
-          </cell>
-          <cell r="D7">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="C8">
-            <v>65</v>
-          </cell>
-          <cell r="D8">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="C9">
-            <v>85</v>
-          </cell>
-          <cell r="D9">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="C10">
-            <v>94</v>
-          </cell>
-          <cell r="D10">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="C11">
-            <v>95</v>
-          </cell>
-          <cell r="D11">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="C12">
-            <v>98</v>
-          </cell>
-          <cell r="D12">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="C13">
-            <v>99</v>
-          </cell>
-          <cell r="D13">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="C14">
-            <v>100</v>
-          </cell>
-          <cell r="D14">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="C15">
-            <v>102</v>
-          </cell>
-          <cell r="D15">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="C16">
-            <v>110</v>
-          </cell>
-          <cell r="D16">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="C17">
-            <v>121</v>
-          </cell>
-          <cell r="D17">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="C18">
-            <v>141</v>
-          </cell>
-          <cell r="D18">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="C19">
-            <v>163</v>
-          </cell>
-          <cell r="D19">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="C20">
-            <v>164</v>
-          </cell>
-          <cell r="D20">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="C21">
-            <v>172</v>
-          </cell>
-          <cell r="D21">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="C22">
-            <v>173</v>
-          </cell>
-          <cell r="D22">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="C23">
-            <v>179</v>
-          </cell>
-          <cell r="D23">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="C24">
-            <v>182</v>
-          </cell>
-          <cell r="D24">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="C25">
-            <v>30</v>
-          </cell>
-          <cell r="D25">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="C26">
-            <v>31</v>
-          </cell>
-          <cell r="D26">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="C27">
-            <v>46</v>
-          </cell>
-          <cell r="D27">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="C28">
-            <v>50</v>
-          </cell>
-          <cell r="D28">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="C29">
-            <v>51</v>
-          </cell>
-          <cell r="D29">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="C30">
-            <v>52</v>
-          </cell>
-          <cell r="D30">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="C31">
-            <v>65</v>
-          </cell>
-          <cell r="D31">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="C32">
-            <v>85</v>
-          </cell>
-          <cell r="D32">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="C33">
-            <v>94</v>
-          </cell>
-          <cell r="D33">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="C34">
-            <v>95</v>
-          </cell>
-          <cell r="D34">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="C35">
-            <v>98</v>
-          </cell>
-          <cell r="D35">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="C36">
-            <v>99</v>
-          </cell>
-          <cell r="D36">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="C37">
-            <v>100</v>
-          </cell>
-          <cell r="D37">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="C38">
-            <v>102</v>
-          </cell>
-          <cell r="D38">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="C39">
-            <v>110</v>
-          </cell>
-          <cell r="D39">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="C40">
-            <v>121</v>
-          </cell>
-          <cell r="D40">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="C41">
-            <v>141</v>
-          </cell>
-          <cell r="D41">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="C42">
-            <v>163</v>
-          </cell>
-          <cell r="D42">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="C43">
-            <v>172</v>
-          </cell>
-          <cell r="D43">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="44">
-          <cell r="C44">
-            <v>173</v>
-          </cell>
-          <cell r="D44">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="45">
-          <cell r="C45">
-            <v>182</v>
-          </cell>
-          <cell r="D45">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="46">
-          <cell r="C46">
-            <v>31</v>
-          </cell>
-          <cell r="D46">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="47">
-          <cell r="C47">
-            <v>46</v>
-          </cell>
-          <cell r="D47">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="48">
-          <cell r="C48">
-            <v>50</v>
-          </cell>
-          <cell r="D48">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="49">
-          <cell r="C49">
-            <v>51</v>
-          </cell>
-          <cell r="D49">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="50">
-          <cell r="C50">
-            <v>52</v>
-          </cell>
-          <cell r="D50">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="51">
-          <cell r="C51">
-            <v>65</v>
-          </cell>
-          <cell r="D51">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="52">
-          <cell r="C52">
-            <v>85</v>
-          </cell>
-          <cell r="D52">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="53">
-          <cell r="C53">
-            <v>94</v>
-          </cell>
-          <cell r="D53">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="C54">
-            <v>95</v>
-          </cell>
-          <cell r="D54">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="55">
-          <cell r="C55">
-            <v>98</v>
-          </cell>
-          <cell r="D55">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="56">
-          <cell r="C56">
-            <v>99</v>
-          </cell>
-          <cell r="D56">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="57">
-          <cell r="C57">
-            <v>100</v>
-          </cell>
-          <cell r="D57">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="58">
-          <cell r="C58">
-            <v>102</v>
-          </cell>
-          <cell r="D58">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="59">
-          <cell r="C59">
-            <v>110</v>
-          </cell>
-          <cell r="D59">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="60">
-          <cell r="C60">
-            <v>121</v>
-          </cell>
-          <cell r="D60">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="61">
-          <cell r="C61">
-            <v>141</v>
-          </cell>
-          <cell r="D61">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="62">
-          <cell r="C62">
-            <v>163</v>
-          </cell>
-          <cell r="D62">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="63">
-          <cell r="C63">
-            <v>31</v>
-          </cell>
-          <cell r="D63">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="64">
-          <cell r="C64">
-            <v>46</v>
-          </cell>
-          <cell r="D64">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="65">
-          <cell r="C65">
-            <v>50</v>
-          </cell>
-          <cell r="D65">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="66">
-          <cell r="C66">
-            <v>51</v>
-          </cell>
-          <cell r="D66">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="67">
-          <cell r="C67">
-            <v>52</v>
-          </cell>
-          <cell r="D67">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="68">
-          <cell r="C68">
-            <v>65</v>
-          </cell>
-          <cell r="D68">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="69">
-          <cell r="C69">
-            <v>85</v>
-          </cell>
-          <cell r="D69">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="70">
-          <cell r="C70">
-            <v>94</v>
-          </cell>
-          <cell r="D70">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="71">
-          <cell r="C71">
-            <v>95</v>
-          </cell>
-          <cell r="D71">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="72">
-          <cell r="C72">
-            <v>98</v>
-          </cell>
-          <cell r="D72">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="73">
-          <cell r="C73">
-            <v>99</v>
-          </cell>
-          <cell r="D73">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="74">
-          <cell r="C74">
-            <v>100</v>
-          </cell>
-          <cell r="D74">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="75">
-          <cell r="C75">
-            <v>102</v>
-          </cell>
-          <cell r="D75">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="76">
-          <cell r="C76">
-            <v>110</v>
-          </cell>
-          <cell r="D76">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="77">
-          <cell r="C77">
-            <v>121</v>
-          </cell>
-          <cell r="D77">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="78">
-          <cell r="C78">
-            <v>141</v>
-          </cell>
-          <cell r="D78">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="79">
-          <cell r="C79">
-            <v>31</v>
-          </cell>
-          <cell r="D79">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="80">
-          <cell r="C80">
-            <v>46</v>
-          </cell>
-          <cell r="D80">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="81">
-          <cell r="C81">
-            <v>50</v>
-          </cell>
-          <cell r="D81">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="82">
-          <cell r="C82">
-            <v>51</v>
-          </cell>
-          <cell r="D82">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="83">
-          <cell r="C83">
-            <v>65</v>
-          </cell>
-          <cell r="D83">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="84">
-          <cell r="C84">
-            <v>85</v>
-          </cell>
-          <cell r="D84">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="85">
-          <cell r="C85">
-            <v>94</v>
-          </cell>
-          <cell r="D85">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="86">
-          <cell r="C86">
-            <v>95</v>
-          </cell>
-          <cell r="D86">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="87">
-          <cell r="C87">
-            <v>98</v>
-          </cell>
-          <cell r="D87">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="88">
-          <cell r="C88">
-            <v>100</v>
-          </cell>
-          <cell r="D88">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="89">
-          <cell r="C89">
-            <v>102</v>
-          </cell>
-          <cell r="D89">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="90">
-          <cell r="C90">
-            <v>110</v>
-          </cell>
-          <cell r="D90">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="91">
-          <cell r="C91">
-            <v>121</v>
-          </cell>
-          <cell r="D91">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="92">
-          <cell r="C92">
-            <v>141</v>
-          </cell>
-          <cell r="D92">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="93">
-          <cell r="C93">
-            <v>31</v>
-          </cell>
-          <cell r="D93">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="94">
-          <cell r="C94">
-            <v>46</v>
-          </cell>
-          <cell r="D94">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="95">
-          <cell r="C95">
-            <v>50</v>
-          </cell>
-          <cell r="D95">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="96">
-          <cell r="C96">
-            <v>51</v>
-          </cell>
-          <cell r="D96">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="97">
-          <cell r="C97">
-            <v>65</v>
-          </cell>
-          <cell r="D97">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="98">
-          <cell r="C98">
-            <v>85</v>
-          </cell>
-          <cell r="D98">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="99">
-          <cell r="C99">
-            <v>95</v>
-          </cell>
-          <cell r="D99">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="100">
-          <cell r="C100">
-            <v>98</v>
-          </cell>
-          <cell r="D100">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="101">
-          <cell r="C101">
-            <v>100</v>
-          </cell>
-          <cell r="D101">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="102">
-          <cell r="C102">
-            <v>102</v>
-          </cell>
-          <cell r="D102">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="103">
-          <cell r="C103">
-            <v>110</v>
-          </cell>
-          <cell r="D103">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="104">
-          <cell r="C104">
-            <v>121</v>
-          </cell>
-          <cell r="D104">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="105">
-          <cell r="C105">
-            <v>31</v>
-          </cell>
-          <cell r="D105">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="106">
-          <cell r="C106">
-            <v>46</v>
-          </cell>
-          <cell r="D106">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="107">
-          <cell r="C107">
-            <v>50</v>
-          </cell>
-          <cell r="D107">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="108">
-          <cell r="C108">
-            <v>51</v>
-          </cell>
-          <cell r="D108">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="109">
-          <cell r="C109">
-            <v>65</v>
-          </cell>
-          <cell r="D109">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="110">
-          <cell r="C110">
-            <v>85</v>
-          </cell>
-          <cell r="D110">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="111">
-          <cell r="C111">
-            <v>95</v>
-          </cell>
-          <cell r="D111">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="112">
-          <cell r="C112">
-            <v>98</v>
-          </cell>
-          <cell r="D112">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="113">
-          <cell r="C113">
-            <v>100</v>
-          </cell>
-          <cell r="D113">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="114">
-          <cell r="C114">
-            <v>102</v>
-          </cell>
-          <cell r="D114">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="115">
-          <cell r="C115">
-            <v>110</v>
-          </cell>
-          <cell r="D115">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="116">
-          <cell r="C116">
-            <v>31</v>
-          </cell>
-          <cell r="D116">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="117">
-          <cell r="C117">
-            <v>46</v>
-          </cell>
-          <cell r="D117">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="118">
-          <cell r="C118">
-            <v>50</v>
-          </cell>
-          <cell r="D118">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="119">
-          <cell r="C119">
-            <v>51</v>
-          </cell>
-          <cell r="D119">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="120">
-          <cell r="C120">
-            <v>65</v>
-          </cell>
-          <cell r="D120">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="121">
-          <cell r="C121">
-            <v>85</v>
-          </cell>
-          <cell r="D121">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="122">
-          <cell r="C122">
-            <v>95</v>
-          </cell>
-          <cell r="D122">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="123">
-          <cell r="C123">
-            <v>98</v>
-          </cell>
-          <cell r="D123">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="124">
-          <cell r="C124">
-            <v>100</v>
-          </cell>
-          <cell r="D124">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="125">
-          <cell r="C125">
-            <v>102</v>
-          </cell>
-          <cell r="D125">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="126">
-          <cell r="C126">
-            <v>31</v>
-          </cell>
-          <cell r="D126">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="127">
-          <cell r="C127">
-            <v>50</v>
-          </cell>
-          <cell r="D127">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="128">
-          <cell r="C128">
-            <v>65</v>
-          </cell>
-          <cell r="D128">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="129">
-          <cell r="C129">
-            <v>85</v>
-          </cell>
-          <cell r="D129">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="130">
-          <cell r="C130">
-            <v>95</v>
-          </cell>
-          <cell r="D130">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="131">
-          <cell r="C131">
-            <v>98</v>
-          </cell>
-          <cell r="D131">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="132">
-          <cell r="C132">
-            <v>100</v>
-          </cell>
-          <cell r="D132">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="133">
-          <cell r="C133">
-            <v>31</v>
-          </cell>
-          <cell r="D133">
-            <v>10</v>
-          </cell>
-        </row>
-        <row r="134">
-          <cell r="C134">
-            <v>50</v>
-          </cell>
-          <cell r="D134">
-            <v>10</v>
-          </cell>
-        </row>
-        <row r="135">
-          <cell r="C135">
-            <v>65</v>
-          </cell>
-          <cell r="D135">
-            <v>10</v>
-          </cell>
-        </row>
-        <row r="136">
-          <cell r="C136">
-            <v>85</v>
-          </cell>
-          <cell r="D136">
-            <v>10</v>
-          </cell>
-        </row>
-        <row r="137">
-          <cell r="C137">
-            <v>31</v>
-          </cell>
-          <cell r="D137">
-            <v>11</v>
-          </cell>
-        </row>
-        <row r="138">
-          <cell r="C138">
-            <v>65</v>
-          </cell>
-          <cell r="D138">
-            <v>11</v>
-          </cell>
-        </row>
-        <row r="139">
-          <cell r="C139">
-            <v>31</v>
-          </cell>
-          <cell r="D139">
-            <v>12</v>
-          </cell>
-        </row>
-        <row r="140">
-          <cell r="C140">
-            <v>31</v>
-          </cell>
-          <cell r="D140">
-            <v>13</v>
-          </cell>
-        </row>
-        <row r="141">
-          <cell r="C141">
-            <v>31</v>
-          </cell>
-          <cell r="D141">
-            <v>14</v>
-          </cell>
-        </row>
-        <row r="142">
-          <cell r="C142">
-            <v>11</v>
-          </cell>
-          <cell r="D142">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="143">
-          <cell r="C143">
-            <v>11</v>
-          </cell>
-          <cell r="D143">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="144">
-          <cell r="C144">
-            <v>11</v>
-          </cell>
-          <cell r="D144">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="145">
-          <cell r="C145">
-            <v>11</v>
-          </cell>
-          <cell r="D145">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="146">
-          <cell r="C146">
-            <v>11</v>
-          </cell>
-          <cell r="D146">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="147">
-          <cell r="C147">
-            <v>11</v>
-          </cell>
-          <cell r="D147">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="148">
-          <cell r="C148">
-            <v>11</v>
-          </cell>
-          <cell r="D148">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="149">
-          <cell r="C149">
-            <v>11</v>
-          </cell>
-          <cell r="D149">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="150">
-          <cell r="C150">
-            <v>11</v>
-          </cell>
-          <cell r="D150">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="151">
-          <cell r="C151">
-            <v>11</v>
-          </cell>
-          <cell r="D151">
-            <v>10</v>
-          </cell>
-        </row>
-        <row r="152">
-          <cell r="C152">
-            <v>11</v>
-          </cell>
-          <cell r="D152">
-            <v>11</v>
-          </cell>
-        </row>
-        <row r="153">
-          <cell r="C153">
-            <v>14</v>
-          </cell>
-          <cell r="D153">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="154">
-          <cell r="C154">
-            <v>14</v>
-          </cell>
-          <cell r="D154">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="155">
-          <cell r="C155">
-            <v>14</v>
-          </cell>
-          <cell r="D155">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="156">
-          <cell r="C156">
-            <v>14</v>
-          </cell>
-          <cell r="D156">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="157">
-          <cell r="C157">
-            <v>14</v>
-          </cell>
-          <cell r="D157">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="158">
-          <cell r="C158">
-            <v>14</v>
-          </cell>
-          <cell r="D158">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="159">
-          <cell r="C159">
-            <v>14</v>
-          </cell>
-          <cell r="D159">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="160">
-          <cell r="C160">
-            <v>14</v>
-          </cell>
-          <cell r="D160">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="161">
-          <cell r="C161">
-            <v>30</v>
-          </cell>
-          <cell r="D161">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="162">
-          <cell r="C162">
-            <v>30</v>
-          </cell>
-          <cell r="D162">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="163">
-          <cell r="C163">
-            <v>30</v>
-          </cell>
-          <cell r="D163">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="164">
-          <cell r="C164">
-            <v>30</v>
-          </cell>
-          <cell r="D164">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="165">
-          <cell r="C165">
-            <v>30</v>
-          </cell>
-          <cell r="D165">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="166">
-          <cell r="C166">
-            <v>30</v>
-          </cell>
-          <cell r="D166">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="167">
-          <cell r="C167">
-            <v>30</v>
-          </cell>
-          <cell r="D167">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="168">
-          <cell r="C168">
-            <v>30</v>
-          </cell>
-          <cell r="D168">
-            <v>10</v>
-          </cell>
-        </row>
-        <row r="169">
-          <cell r="C169">
-            <v>30</v>
-          </cell>
-          <cell r="D169">
-            <v>11</v>
-          </cell>
-        </row>
-        <row r="170">
-          <cell r="C170">
-            <v>33</v>
-          </cell>
-          <cell r="D170">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="171">
-          <cell r="C171">
-            <v>33</v>
-          </cell>
-          <cell r="D171">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="172">
-          <cell r="C172">
-            <v>33</v>
-          </cell>
-          <cell r="D172">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="173">
-          <cell r="C173">
-            <v>33</v>
-          </cell>
-          <cell r="D173">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="174">
-          <cell r="C174">
-            <v>33</v>
-          </cell>
-          <cell r="D174">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="175">
-          <cell r="C175">
-            <v>33</v>
-          </cell>
-          <cell r="D175">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="176">
-          <cell r="C176">
-            <v>33</v>
-          </cell>
-          <cell r="D176">
-            <v>10</v>
-          </cell>
-        </row>
-        <row r="177">
-          <cell r="C177">
-            <v>33</v>
-          </cell>
-          <cell r="D177">
-            <v>11</v>
-          </cell>
-        </row>
-        <row r="178">
-          <cell r="C178">
-            <v>33</v>
-          </cell>
-          <cell r="D178">
-            <v>12</v>
-          </cell>
-        </row>
-        <row r="179">
-          <cell r="C179">
-            <v>33</v>
-          </cell>
-          <cell r="D179">
-            <v>13</v>
-          </cell>
-        </row>
-        <row r="180">
-          <cell r="C180">
-            <v>33</v>
-          </cell>
-          <cell r="D180">
-            <v>14</v>
-          </cell>
-        </row>
-        <row r="181">
-          <cell r="C181">
-            <v>33</v>
-          </cell>
-          <cell r="D181">
-            <v>15</v>
-          </cell>
-        </row>
-        <row r="182">
-          <cell r="C182">
-            <v>91</v>
-          </cell>
-          <cell r="D182">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="183">
-          <cell r="C183">
-            <v>91</v>
-          </cell>
-          <cell r="D183">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="184">
-          <cell r="C184">
-            <v>91</v>
-          </cell>
-          <cell r="D184">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="185">
-          <cell r="C185">
-            <v>91</v>
-          </cell>
-          <cell r="D185">
-            <v>4</v>
-          </cell>
-        </row>
-        <row r="186">
-          <cell r="C186">
-            <v>91</v>
-          </cell>
-          <cell r="D186">
-            <v>5</v>
-          </cell>
-        </row>
-        <row r="187">
-          <cell r="C187">
-            <v>103</v>
-          </cell>
-          <cell r="D187">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="188">
-          <cell r="C188">
-            <v>107</v>
-          </cell>
-          <cell r="D188">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="189">
-          <cell r="C189">
-            <v>107</v>
-          </cell>
-          <cell r="D189">
-            <v>2</v>
-          </cell>
-        </row>
-        <row r="190">
-          <cell r="C190">
-            <v>150</v>
-          </cell>
-          <cell r="D190">
-            <v>1</v>
-          </cell>
-        </row>
-        <row r="191">
-          <cell r="C191">
-            <v>11</v>
-          </cell>
-          <cell r="D191">
-            <v>12</v>
-          </cell>
-        </row>
-        <row r="192">
-          <cell r="C192">
-            <v>14</v>
-          </cell>
-          <cell r="D192">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="193">
-          <cell r="C193">
-            <v>30</v>
-          </cell>
-          <cell r="D193">
-            <v>12</v>
-          </cell>
-        </row>
-        <row r="194">
-          <cell r="C194">
-            <v>33</v>
-          </cell>
-          <cell r="D194">
-            <v>16</v>
-          </cell>
-        </row>
-        <row r="195">
-          <cell r="C195">
-            <v>107</v>
-          </cell>
-          <cell r="D195">
-            <v>3</v>
-          </cell>
-        </row>
-        <row r="196">
-          <cell r="C196">
-            <v>91</v>
-          </cell>
-          <cell r="D196">
-            <v>6</v>
-          </cell>
-        </row>
-        <row r="197">
-          <cell r="C197">
-            <v>11</v>
-          </cell>
-          <cell r="D197">
-            <v>13</v>
-          </cell>
-        </row>
-        <row r="198">
-          <cell r="C198">
-            <v>91</v>
-          </cell>
-          <cell r="D198">
-            <v>7</v>
-          </cell>
-        </row>
-        <row r="199">
-          <cell r="C199">
-            <v>33</v>
-          </cell>
-          <cell r="D199">
-            <v>17</v>
-          </cell>
-        </row>
-        <row r="200">
-          <cell r="C200">
-            <v>30</v>
-          </cell>
-          <cell r="D200">
-            <v>13</v>
-          </cell>
-        </row>
-        <row r="201">
-          <cell r="C201">
-            <v>14</v>
-          </cell>
-          <cell r="D201">
-            <v>10</v>
-          </cell>
-        </row>
-        <row r="202">
-          <cell r="C202">
-            <v>11</v>
-          </cell>
-          <cell r="D202">
-            <v>14</v>
-          </cell>
-        </row>
-        <row r="203">
-          <cell r="C203">
-            <v>91</v>
-          </cell>
-          <cell r="D203">
-            <v>8</v>
-          </cell>
-        </row>
-        <row r="204">
-          <cell r="C204">
-            <v>33</v>
-          </cell>
-          <cell r="D204">
-            <v>18</v>
-          </cell>
-        </row>
-        <row r="205">
-          <cell r="C205">
-            <v>30</v>
-          </cell>
-          <cell r="D205">
-            <v>14</v>
-          </cell>
-        </row>
-        <row r="206">
-          <cell r="C206">
-            <v>14</v>
-          </cell>
-          <cell r="D206">
-            <v>11</v>
-          </cell>
-        </row>
-        <row r="207">
-          <cell r="C207">
-            <v>11</v>
-          </cell>
-          <cell r="D207">
-            <v>15</v>
-          </cell>
-        </row>
-        <row r="208">
-          <cell r="C208">
-            <v>14</v>
-          </cell>
-          <cell r="D208">
-            <v>12</v>
-          </cell>
-        </row>
-        <row r="209">
-          <cell r="C209">
-            <v>91</v>
-          </cell>
-          <cell r="D209">
-            <v>9</v>
-          </cell>
-        </row>
-        <row r="210">
-          <cell r="C210">
-            <v>33</v>
-          </cell>
-          <cell r="D210">
-            <v>19</v>
-          </cell>
-        </row>
-        <row r="211">
-          <cell r="C211">
-            <v>30</v>
-          </cell>
-          <cell r="D211">
-            <v>15</v>
-          </cell>
-        </row>
-        <row r="212">
-          <cell r="C212">
-            <v>150</v>
-          </cell>
-          <cell r="D212">
-            <v>2</v>
+          <cell r="B1" t="str">
+            <v>ID</v>
           </cell>
         </row>
       </sheetData>
@@ -4352,13 +2655,7 @@
         </row>
       </sheetData>
       <sheetData sheetId="9"/>
-      <sheetData sheetId="10">
-        <row r="1">
-          <cell r="G1" t="str">
-            <v>unit</v>
-          </cell>
-        </row>
-      </sheetData>
+      <sheetData sheetId="10"/>
       <sheetData sheetId="11"/>
       <sheetData sheetId="12"/>
       <sheetData sheetId="13"/>
@@ -4682,7 +2979,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr codeName="Sheet1" filterMode="1"/>
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AW87"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
@@ -4694,15 +2991,15 @@
     <col min="7" max="7" width="15.140625" style="5" customWidth="1"/>
     <col min="8" max="8" width="3" customWidth="1"/>
     <col min="9" max="9" width="4.42578125" style="78" customWidth="1"/>
-    <col min="10" max="10" width="6.140625" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="11" max="13" width="8.28515625" hidden="1" customWidth="1" outlineLevel="2"/>
-    <col min="14" max="14" width="12.85546875" style="5" hidden="1" customWidth="1" outlineLevel="2"/>
-    <col min="15" max="15" width="18.28515625" style="5" hidden="1" customWidth="1" outlineLevel="2"/>
-    <col min="16" max="16" width="13.140625" style="60" hidden="1" customWidth="1" outlineLevel="2"/>
-    <col min="17" max="17" width="12.7109375" hidden="1" customWidth="1" outlineLevel="2"/>
-    <col min="18" max="18" width="15.7109375" hidden="1" customWidth="1" outlineLevel="2"/>
-    <col min="19" max="19" width="28.140625" hidden="1" customWidth="1" outlineLevel="2"/>
-    <col min="20" max="20" width="4" customWidth="1" collapsed="1"/>
+    <col min="10" max="10" width="6.140625" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="13" width="8.28515625" customWidth="1" outlineLevel="2"/>
+    <col min="14" max="14" width="12.85546875" style="5" customWidth="1" outlineLevel="2"/>
+    <col min="15" max="15" width="18.28515625" style="5" customWidth="1" outlineLevel="2"/>
+    <col min="16" max="16" width="13.140625" style="60" customWidth="1" outlineLevel="2"/>
+    <col min="17" max="17" width="12.7109375" customWidth="1" outlineLevel="2"/>
+    <col min="18" max="18" width="15.7109375" customWidth="1" outlineLevel="2"/>
+    <col min="19" max="19" width="28.140625" customWidth="1" outlineLevel="2"/>
+    <col min="20" max="20" width="4" customWidth="1"/>
     <col min="21" max="21" width="6.7109375" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="22" max="22" width="9" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="23" max="23" width="10" hidden="1" customWidth="1" outlineLevel="1"/>
@@ -4848,7 +3145,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="2" spans="1:49" hidden="1">
+    <row r="2" spans="1:49">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5174,7 +3471,7 @@
       <c r="AV4" s="1"/>
       <c r="AW4" s="1"/>
     </row>
-    <row r="5" spans="1:49" hidden="1">
+    <row r="5" spans="1:49">
       <c r="A5">
         <f t="shared" si="3"/>
         <v>4</v>
@@ -5357,7 +3654,7 @@
       <c r="AV6" s="1"/>
       <c r="AW6" s="1"/>
     </row>
-    <row r="7" spans="1:49" hidden="1">
+    <row r="7" spans="1:49">
       <c r="A7">
         <f t="shared" si="3"/>
         <v>6</v>
@@ -5571,7 +3868,7 @@
       <c r="AV8" s="1"/>
       <c r="AW8" s="1"/>
     </row>
-    <row r="9" spans="1:49" hidden="1">
+    <row r="9" spans="1:49">
       <c r="A9">
         <f t="shared" si="3"/>
         <v>8</v>
@@ -5670,7 +3967,7 @@
       <c r="AV9" s="1"/>
       <c r="AW9" s="1"/>
     </row>
-    <row r="10" spans="1:49" hidden="1">
+    <row r="10" spans="1:49">
       <c r="A10">
         <f t="shared" si="3"/>
         <v>9</v>
@@ -5755,7 +4052,7 @@
       <c r="AV10" s="1"/>
       <c r="AW10" s="1"/>
     </row>
-    <row r="11" spans="1:49" hidden="1">
+    <row r="11" spans="1:49">
       <c r="A11">
         <f t="shared" si="3"/>
         <v>10</v>
@@ -5840,7 +4137,7 @@
       <c r="AV11" s="1"/>
       <c r="AW11" s="1"/>
     </row>
-    <row r="12" spans="1:49" hidden="1">
+    <row r="12" spans="1:49">
       <c r="A12">
         <f t="shared" si="3"/>
         <v>11</v>
@@ -5925,7 +4222,7 @@
       <c r="AV12" s="1"/>
       <c r="AW12" s="1"/>
     </row>
-    <row r="13" spans="1:49" hidden="1">
+    <row r="13" spans="1:49">
       <c r="A13">
         <f t="shared" si="3"/>
         <v>12</v>
@@ -6013,7 +4310,7 @@
       <c r="AV13" s="1"/>
       <c r="AW13" s="1"/>
     </row>
-    <row r="14" spans="1:49" hidden="1">
+    <row r="14" spans="1:49">
       <c r="A14">
         <f t="shared" si="3"/>
         <v>13</v>
@@ -6098,7 +4395,7 @@
       <c r="AV14" s="1"/>
       <c r="AW14" s="1"/>
     </row>
-    <row r="15" spans="1:49" hidden="1">
+    <row r="15" spans="1:49">
       <c r="A15">
         <f t="shared" si="3"/>
         <v>14</v>
@@ -6180,7 +4477,7 @@
       <c r="AV15" s="1"/>
       <c r="AW15" s="1"/>
     </row>
-    <row r="16" spans="1:49" hidden="1">
+    <row r="16" spans="1:49">
       <c r="A16">
         <f t="shared" si="3"/>
         <v>15</v>
@@ -6301,7 +4598,7 @@
       <c r="AV16" s="1"/>
       <c r="AW16" s="1"/>
     </row>
-    <row r="17" spans="1:49" hidden="1">
+    <row r="17" spans="1:49">
       <c r="A17">
         <f t="shared" si="3"/>
         <v>16</v>
@@ -6423,7 +4720,7 @@
       <c r="AV17" s="1"/>
       <c r="AW17" s="1"/>
     </row>
-    <row r="18" spans="1:49" hidden="1">
+    <row r="18" spans="1:49">
       <c r="A18">
         <f t="shared" si="3"/>
         <v>17</v>
@@ -6510,7 +4807,7 @@
       <c r="AV18" s="1"/>
       <c r="AW18" s="1"/>
     </row>
-    <row r="19" spans="1:49" hidden="1">
+    <row r="19" spans="1:49">
       <c r="A19">
         <f t="shared" si="3"/>
         <v>18</v>
@@ -6589,7 +4886,7 @@
       <c r="AV19" s="1"/>
       <c r="AW19" s="1"/>
     </row>
-    <row r="20" spans="1:49" hidden="1">
+    <row r="20" spans="1:49">
       <c r="A20">
         <f t="shared" si="3"/>
         <v>19</v>
@@ -6676,7 +4973,7 @@
       <c r="AV20" s="1"/>
       <c r="AW20" s="1"/>
     </row>
-    <row r="21" spans="1:49" hidden="1">
+    <row r="21" spans="1:49">
       <c r="A21">
         <f t="shared" si="3"/>
         <v>20</v>
@@ -6776,7 +5073,7 @@
       <c r="AV21" s="1"/>
       <c r="AW21" s="1"/>
     </row>
-    <row r="22" spans="1:49" hidden="1">
+    <row r="22" spans="1:49">
       <c r="A22">
         <f t="shared" si="3"/>
         <v>21</v>
@@ -6876,7 +5173,7 @@
       <c r="AV22" s="1"/>
       <c r="AW22" s="1"/>
     </row>
-    <row r="23" spans="1:49" hidden="1">
+    <row r="23" spans="1:49">
       <c r="A23">
         <f t="shared" si="3"/>
         <v>22</v>
@@ -6976,7 +5273,7 @@
       <c r="AV23" s="1"/>
       <c r="AW23" s="1"/>
     </row>
-    <row r="24" spans="1:49" hidden="1">
+    <row r="24" spans="1:49">
       <c r="A24">
         <f t="shared" si="3"/>
         <v>23</v>
@@ -7065,7 +5362,7 @@
       <c r="AV24" s="1"/>
       <c r="AW24" s="1"/>
     </row>
-    <row r="25" spans="1:49" hidden="1">
+    <row r="25" spans="1:49">
       <c r="A25">
         <f t="shared" si="3"/>
         <v>24</v>
@@ -7143,7 +5440,7 @@
       <c r="AV25" s="1"/>
       <c r="AW25" s="1"/>
     </row>
-    <row r="26" spans="1:49" hidden="1">
+    <row r="26" spans="1:49">
       <c r="A26">
         <f t="shared" si="3"/>
         <v>25</v>
@@ -7262,7 +5559,7 @@
       <c r="AV26" s="1"/>
       <c r="AW26" s="1"/>
     </row>
-    <row r="27" spans="1:49" hidden="1">
+    <row r="27" spans="1:49">
       <c r="A27">
         <f t="shared" si="3"/>
         <v>26</v>
@@ -7350,7 +5647,7 @@
       <c r="AV27" s="1"/>
       <c r="AW27" s="1"/>
     </row>
-    <row r="28" spans="1:49" hidden="1">
+    <row r="28" spans="1:49">
       <c r="A28">
         <f t="shared" si="3"/>
         <v>27</v>
@@ -7471,7 +5768,7 @@
       <c r="AV28" s="1"/>
       <c r="AW28" s="1"/>
     </row>
-    <row r="29" spans="1:49" hidden="1">
+    <row r="29" spans="1:49">
       <c r="A29">
         <f t="shared" si="3"/>
         <v>28</v>
@@ -7590,7 +5887,7 @@
       <c r="AV29" s="1"/>
       <c r="AW29" s="1"/>
     </row>
-    <row r="30" spans="1:49" hidden="1">
+    <row r="30" spans="1:49">
       <c r="A30">
         <f t="shared" si="3"/>
         <v>29</v>
@@ -7684,7 +5981,7 @@
       <c r="AV30" s="1"/>
       <c r="AW30" s="1"/>
     </row>
-    <row r="31" spans="1:49" hidden="1">
+    <row r="31" spans="1:49">
       <c r="A31">
         <f t="shared" si="3"/>
         <v>30</v>
@@ -7767,7 +6064,7 @@
       <c r="AV31" s="1"/>
       <c r="AW31" s="1"/>
     </row>
-    <row r="32" spans="1:49" hidden="1">
+    <row r="32" spans="1:49">
       <c r="A32">
         <f t="shared" si="3"/>
         <v>31</v>
@@ -7886,7 +6183,7 @@
       <c r="AV32" s="1"/>
       <c r="AW32" s="1"/>
     </row>
-    <row r="33" spans="1:49" hidden="1">
+    <row r="33" spans="1:49">
       <c r="A33">
         <f t="shared" si="3"/>
         <v>32</v>
@@ -8008,7 +6305,7 @@
       <c r="AV33" s="1"/>
       <c r="AW33" s="1"/>
     </row>
-    <row r="34" spans="1:49" hidden="1">
+    <row r="34" spans="1:49">
       <c r="A34">
         <f t="shared" si="3"/>
         <v>33</v>
@@ -8103,7 +6400,7 @@
       <c r="AV34" s="1"/>
       <c r="AW34" s="1"/>
     </row>
-    <row r="35" spans="1:49" hidden="1">
+    <row r="35" spans="1:49">
       <c r="A35">
         <f t="shared" si="3"/>
         <v>34</v>
@@ -8222,7 +6519,7 @@
       <c r="AV35" s="1"/>
       <c r="AW35" s="1"/>
     </row>
-    <row r="36" spans="1:49" hidden="1">
+    <row r="36" spans="1:49">
       <c r="A36">
         <f t="shared" si="3"/>
         <v>35</v>
@@ -8438,7 +6735,7 @@
       <c r="AV37" s="1"/>
       <c r="AW37" s="1"/>
     </row>
-    <row r="38" spans="1:49" hidden="1">
+    <row r="38" spans="1:49">
       <c r="A38">
         <f t="shared" si="3"/>
         <v>37</v>
@@ -8521,7 +6818,7 @@
       <c r="AV38" s="1"/>
       <c r="AW38" s="1"/>
     </row>
-    <row r="39" spans="1:49" hidden="1">
+    <row r="39" spans="1:49">
       <c r="A39">
         <f t="shared" si="3"/>
         <v>38</v>
@@ -8618,7 +6915,7 @@
       <c r="AV39" s="1"/>
       <c r="AW39" s="1"/>
     </row>
-    <row r="40" spans="1:49" hidden="1">
+    <row r="40" spans="1:49">
       <c r="A40">
         <f t="shared" si="3"/>
         <v>39</v>
@@ -8715,7 +7012,7 @@
       <c r="AV40" s="1"/>
       <c r="AW40" s="1"/>
     </row>
-    <row r="41" spans="1:49" hidden="1">
+    <row r="41" spans="1:49">
       <c r="A41">
         <f t="shared" si="3"/>
         <v>40</v>
@@ -8801,7 +7098,7 @@
       <c r="AV41" s="1"/>
       <c r="AW41" s="1"/>
     </row>
-    <row r="42" spans="1:49" hidden="1">
+    <row r="42" spans="1:49">
       <c r="A42">
         <f t="shared" si="3"/>
         <v>41</v>
@@ -8894,7 +7191,7 @@
       <c r="AV42" s="1"/>
       <c r="AW42" s="1"/>
     </row>
-    <row r="43" spans="1:49" hidden="1">
+    <row r="43" spans="1:49">
       <c r="A43">
         <f t="shared" si="3"/>
         <v>42</v>
@@ -8995,7 +7292,7 @@
       <c r="AV43" s="1"/>
       <c r="AW43" s="1"/>
     </row>
-    <row r="44" spans="1:49" hidden="1">
+    <row r="44" spans="1:49">
       <c r="A44">
         <f t="shared" si="3"/>
         <v>43</v>
@@ -9081,7 +7378,7 @@
       <c r="AV44" s="1"/>
       <c r="AW44" s="1"/>
     </row>
-    <row r="45" spans="1:49" hidden="1">
+    <row r="45" spans="1:49">
       <c r="A45">
         <f t="shared" si="3"/>
         <v>44</v>
@@ -9203,7 +7500,7 @@
       <c r="AV45" s="1"/>
       <c r="AW45" s="1"/>
     </row>
-    <row r="46" spans="1:49" hidden="1">
+    <row r="46" spans="1:49">
       <c r="A46">
         <f t="shared" si="3"/>
         <v>45</v>
@@ -9289,7 +7586,7 @@
       <c r="AV46" s="1"/>
       <c r="AW46" s="1"/>
     </row>
-    <row r="47" spans="1:49" hidden="1">
+    <row r="47" spans="1:49">
       <c r="A47">
         <f t="shared" si="3"/>
         <v>46</v>
@@ -9408,7 +7705,7 @@
       <c r="AV47" s="1"/>
       <c r="AW47" s="1"/>
     </row>
-    <row r="48" spans="1:49" hidden="1">
+    <row r="48" spans="1:49">
       <c r="A48">
         <f t="shared" si="3"/>
         <v>47</v>
@@ -9522,7 +7819,7 @@
       <c r="AV48" s="1"/>
       <c r="AW48" s="1"/>
     </row>
-    <row r="49" spans="1:49" hidden="1">
+    <row r="49" spans="1:49">
       <c r="A49">
         <f t="shared" si="3"/>
         <v>48</v>
@@ -9640,7 +7937,7 @@
       <c r="AV49" s="1"/>
       <c r="AW49" s="1"/>
     </row>
-    <row r="50" spans="1:49" hidden="1">
+    <row r="50" spans="1:49">
       <c r="A50">
         <f t="shared" si="3"/>
         <v>49</v>
@@ -9762,7 +8059,7 @@
       <c r="AV50" s="1"/>
       <c r="AW50" s="1"/>
     </row>
-    <row r="51" spans="1:49" hidden="1">
+    <row r="51" spans="1:49">
       <c r="A51">
         <f t="shared" si="3"/>
         <v>50</v>
@@ -9864,7 +8161,7 @@
       <c r="AV51" s="1"/>
       <c r="AW51" s="1"/>
     </row>
-    <row r="52" spans="1:49" hidden="1">
+    <row r="52" spans="1:49">
       <c r="A52">
         <f t="shared" si="3"/>
         <v>51</v>
@@ -9966,7 +8263,7 @@
       <c r="AV52" s="1"/>
       <c r="AW52" s="1"/>
     </row>
-    <row r="53" spans="1:49" hidden="1">
+    <row r="53" spans="1:49">
       <c r="A53">
         <f t="shared" si="3"/>
         <v>52</v>
@@ -10085,7 +8382,7 @@
       <c r="AV53" s="1"/>
       <c r="AW53" s="1"/>
     </row>
-    <row r="54" spans="1:49" hidden="1">
+    <row r="54" spans="1:49">
       <c r="A54">
         <f t="shared" si="3"/>
         <v>53</v>
@@ -10204,7 +8501,7 @@
       <c r="AV54" s="1"/>
       <c r="AW54" s="1"/>
     </row>
-    <row r="55" spans="1:49" hidden="1">
+    <row r="55" spans="1:49">
       <c r="A55">
         <f t="shared" si="3"/>
         <v>54</v>
@@ -10326,7 +8623,7 @@
       <c r="AV55" s="1"/>
       <c r="AW55" s="1"/>
     </row>
-    <row r="56" spans="1:49" hidden="1">
+    <row r="56" spans="1:49">
       <c r="A56">
         <f t="shared" si="3"/>
         <v>55</v>
@@ -10424,7 +8721,7 @@
       <c r="AV56" s="1"/>
       <c r="AW56" s="1"/>
     </row>
-    <row r="57" spans="1:49" hidden="1">
+    <row r="57" spans="1:49">
       <c r="A57">
         <f t="shared" si="3"/>
         <v>56</v>
@@ -10530,7 +8827,7 @@
       <c r="AV57" s="1"/>
       <c r="AW57" s="1"/>
     </row>
-    <row r="58" spans="1:49" hidden="1">
+    <row r="58" spans="1:49">
       <c r="A58">
         <f t="shared" si="3"/>
         <v>57</v>
@@ -10606,7 +8903,7 @@
       <c r="AV58" s="1"/>
       <c r="AW58" s="1"/>
     </row>
-    <row r="59" spans="1:49" hidden="1">
+    <row r="59" spans="1:49">
       <c r="A59">
         <f t="shared" si="3"/>
         <v>58</v>
@@ -10698,7 +8995,7 @@
       <c r="AV59" s="1"/>
       <c r="AW59" s="1"/>
     </row>
-    <row r="60" spans="1:49" hidden="1">
+    <row r="60" spans="1:49">
       <c r="A60">
         <f t="shared" si="3"/>
         <v>59</v>
@@ -10809,7 +9106,7 @@
       <c r="AV60" s="1"/>
       <c r="AW60" s="1"/>
     </row>
-    <row r="61" spans="1:49" hidden="1">
+    <row r="61" spans="1:49">
       <c r="A61">
         <f t="shared" si="3"/>
         <v>60</v>
@@ -10897,7 +9194,7 @@
       <c r="AV61" s="1"/>
       <c r="AW61" s="1"/>
     </row>
-    <row r="62" spans="1:49" hidden="1">
+    <row r="62" spans="1:49">
       <c r="A62">
         <f t="shared" si="3"/>
         <v>61</v>
@@ -10988,7 +9285,7 @@
       <c r="AV62" s="1"/>
       <c r="AW62" s="1"/>
     </row>
-    <row r="63" spans="1:49" hidden="1">
+    <row r="63" spans="1:49">
       <c r="A63">
         <f t="shared" si="3"/>
         <v>62</v>
@@ -11079,7 +9376,7 @@
       <c r="AV63" s="1"/>
       <c r="AW63" s="1"/>
     </row>
-    <row r="64" spans="1:49" hidden="1">
+    <row r="64" spans="1:49">
       <c r="A64">
         <f t="shared" si="3"/>
         <v>63</v>
@@ -11170,7 +9467,7 @@
       <c r="AV64" s="1"/>
       <c r="AW64" s="1"/>
     </row>
-    <row r="65" spans="1:49" hidden="1">
+    <row r="65" spans="1:49">
       <c r="A65">
         <f t="shared" si="3"/>
         <v>64</v>
@@ -11261,7 +9558,7 @@
       <c r="AV65" s="1"/>
       <c r="AW65" s="1"/>
     </row>
-    <row r="66" spans="1:49" hidden="1">
+    <row r="66" spans="1:49">
       <c r="A66">
         <f t="shared" si="3"/>
         <v>65</v>
@@ -11352,7 +9649,7 @@
       <c r="AV66" s="1"/>
       <c r="AW66" s="1"/>
     </row>
-    <row r="67" spans="1:49" hidden="1">
+    <row r="67" spans="1:49">
       <c r="A67">
         <f t="shared" si="3"/>
         <v>66</v>
@@ -11440,7 +9737,7 @@
       <c r="AV67" s="1"/>
       <c r="AW67" s="1"/>
     </row>
-    <row r="68" spans="1:49" hidden="1">
+    <row r="68" spans="1:49">
       <c r="A68">
         <f t="shared" si="3"/>
         <v>67</v>
@@ -11528,7 +9825,7 @@
       <c r="AV68" s="1"/>
       <c r="AW68" s="1"/>
     </row>
-    <row r="69" spans="1:49" hidden="1">
+    <row r="69" spans="1:49">
       <c r="A69">
         <f t="shared" ref="A69:A87" si="48">+A68+1</f>
         <v>68</v>
@@ -11616,7 +9913,7 @@
       <c r="AV69" s="1"/>
       <c r="AW69" s="1"/>
     </row>
-    <row r="70" spans="1:49" hidden="1">
+    <row r="70" spans="1:49">
       <c r="A70">
         <f t="shared" si="48"/>
         <v>69</v>
@@ -11704,7 +10001,7 @@
       <c r="AV70" s="1"/>
       <c r="AW70" s="1"/>
     </row>
-    <row r="71" spans="1:49" hidden="1">
+    <row r="71" spans="1:49">
       <c r="A71">
         <f t="shared" si="48"/>
         <v>70</v>
@@ -11795,7 +10092,7 @@
       <c r="AV71" s="1"/>
       <c r="AW71" s="1"/>
     </row>
-    <row r="72" spans="1:49" hidden="1">
+    <row r="72" spans="1:49">
       <c r="A72">
         <f t="shared" si="48"/>
         <v>71</v>
@@ -11863,7 +10160,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="73" spans="1:49" hidden="1">
+    <row r="73" spans="1:49">
       <c r="A73">
         <f t="shared" si="48"/>
         <v>72</v>
@@ -11958,7 +10255,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="74" spans="1:49" hidden="1">
+    <row r="74" spans="1:49">
       <c r="A74">
         <f t="shared" si="48"/>
         <v>73</v>
@@ -12039,7 +10336,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="75" spans="1:49" hidden="1">
+    <row r="75" spans="1:49">
       <c r="A75">
         <f t="shared" si="48"/>
         <v>74</v>
@@ -12119,7 +10416,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="76" spans="1:49" hidden="1">
+    <row r="76" spans="1:49">
       <c r="A76">
         <f>+A74+1</f>
         <v>74</v>
@@ -12199,7 +10496,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="77" spans="1:49" hidden="1">
+    <row r="77" spans="1:49">
       <c r="A77">
         <f>+A75+1</f>
         <v>75</v>
@@ -12279,7 +10576,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="78" spans="1:49" hidden="1">
+    <row r="78" spans="1:49">
       <c r="A78">
         <f t="shared" si="48"/>
         <v>76</v>
@@ -12350,7 +10647,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="79" spans="1:49" hidden="1">
+    <row r="79" spans="1:49">
       <c r="A79">
         <f t="shared" si="48"/>
         <v>77</v>
@@ -12418,7 +10715,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="80" spans="1:49" hidden="1">
+    <row r="80" spans="1:49">
       <c r="A80">
         <f t="shared" si="48"/>
         <v>78</v>
@@ -12489,7 +10786,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="81" spans="1:36" hidden="1">
+    <row r="81" spans="1:36">
       <c r="A81">
         <f t="shared" si="48"/>
         <v>79</v>
@@ -12557,7 +10854,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="82" spans="1:36" hidden="1">
+    <row r="82" spans="1:36">
       <c r="A82">
         <f t="shared" si="48"/>
         <v>80</v>
@@ -12628,7 +10925,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="83" spans="1:36" hidden="1">
+    <row r="83" spans="1:36">
       <c r="A83">
         <f t="shared" si="48"/>
         <v>81</v>
@@ -12732,7 +11029,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="84" spans="1:36" hidden="1">
+    <row r="84" spans="1:36">
       <c r="A84">
         <f t="shared" si="48"/>
         <v>82</v>
@@ -12815,7 +11112,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="85" spans="1:36" hidden="1">
+    <row r="85" spans="1:36">
       <c r="A85">
         <f t="shared" si="48"/>
         <v>83</v>
@@ -12910,7 +11207,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="86" spans="1:36" hidden="1">
+    <row r="86" spans="1:36">
       <c r="A86">
         <f t="shared" si="48"/>
         <v>84</v>
@@ -13014,7 +11311,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="87" spans="1:36" hidden="1">
+    <row r="87" spans="1:36">
       <c r="A87">
         <f t="shared" si="48"/>
         <v>85</v>
@@ -13101,26 +11398,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AR87" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="2">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-    <filterColumn colId="9">
-      <filters>
-        <filter val="EB"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="10">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-    <filterColumn colId="35">
-      <filters blank="1"/>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:AR87" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="S2:S46">
     <sortCondition ref="S2:S46"/>
   </sortState>
@@ -13604,7 +11882,7 @@
       <c r="B3" s="90"/>
       <c r="C3" s="84" t="str">
         <f>_xlfn.XLOOKUP(L3,data!L:L,data!F:F,,0)</f>
-        <v>NAR KRAN MMC</v>
+        <v>Əsgərov Yaşar</v>
       </c>
       <c r="D3" s="85"/>
       <c r="E3" s="85"/>
@@ -13619,7 +11897,7 @@
       </c>
       <c r="J3" s="83"/>
       <c r="L3" s="46">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="M3" s="46">
         <v>4</v>
@@ -13629,7 +11907,7 @@
       </c>
       <c r="O3" s="47" t="str">
         <f>_xlfn.XLOOKUP(L3,data!L:L,data!R:R,0)</f>
-        <v>Warehouse</v>
+        <v>Infrastructure</v>
       </c>
       <c r="T3" s="43" t="s">
         <v>116</v>
@@ -13664,7 +11942,7 @@
       <c r="B4" s="14"/>
       <c r="C4" s="84" t="str" cm="1">
         <f t="array" ref="C4">INDEX(_xlfn.TEXTSPLIT(_xlfn.XLOOKUP(L3,data!L:L,data!N:N,,0),"-"),1)</f>
-        <v>99DX853</v>
+        <v>110FA930</v>
       </c>
       <c r="D4" s="85"/>
       <c r="E4" s="85"/>
@@ -13675,14 +11953,14 @@
       <c r="H4" s="91"/>
       <c r="I4" s="100" t="str">
         <f>_xlfn.XLOOKUP(L3,data!L:L,data!D:D,,0)</f>
-        <v>KLN-SPP2-EQ-119</v>
+        <v>KLN-SPP2-EQ-163</v>
       </c>
       <c r="J4" s="83"/>
       <c r="L4" s="66">
         <v>179</v>
       </c>
       <c r="M4" s="65">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N4" s="49"/>
       <c r="O4" s="49"/>
@@ -13717,9 +11995,9 @@
         <v>173</v>
       </c>
       <c r="B5" s="14"/>
-      <c r="C5" s="84">
+      <c r="C5" s="84" t="str">
         <f>_xlfn.XLOOKUP(L3,data!L:L,data!Q:Q,,0)</f>
-        <v>0</v>
+        <v>Komatsu</v>
       </c>
       <c r="D5" s="85"/>
       <c r="E5" s="85"/>
@@ -13777,7 +12055,7 @@
       <c r="H6" s="91"/>
       <c r="I6" s="92" t="str">
         <f>""&amp;MID(_xlfn.XLOOKUP(L3,data!L:L,data!G:G,,0),2,12)</f>
-        <v>994502712731</v>
+        <v>994558864957</v>
       </c>
       <c r="J6" s="93"/>
       <c r="O6" cm="1">
@@ -14724,7 +13002,7 @@
     <row r="41" spans="1:12" ht="31.5" customHeight="1" thickBot="1">
       <c r="A41" s="101" t="str">
         <f>_xlfn.XLOOKUP(L3,data!L:L,data!F:F)</f>
-        <v>NAR KRAN MMC</v>
+        <v>Əsgərov Yaşar</v>
       </c>
       <c r="B41" s="102"/>
       <c r="C41" s="102"/>
@@ -14735,7 +13013,7 @@
       <c r="F41" s="96"/>
       <c r="G41" s="97" t="str">
         <f>A41</f>
-        <v>NAR KRAN MMC</v>
+        <v>Əsgərov Yaşar</v>
       </c>
       <c r="H41" s="98"/>
       <c r="I41" s="99"/>
@@ -14754,7 +13032,7 @@
       <c r="F42" s="96"/>
       <c r="G42" s="97" t="str">
         <f>_xlfn.XLOOKUP(L3,data!L:L,data!M:M)</f>
-        <v>Mustafa Yazıcı</v>
+        <v>Azər Əbilov</v>
       </c>
       <c r="H42" s="98"/>
       <c r="I42" s="99"/>
@@ -14768,13 +13046,13 @@
       <c r="C43" s="42"/>
       <c r="D43" s="94" t="str">
         <f>VLOOKUP(O3,_xlfn._TRO_TRAILING(T:V),2,0)</f>
-        <v>Ambar şefi</v>
+        <v>Alt yapı ve Harita şefi</v>
       </c>
       <c r="E43" s="95"/>
       <c r="F43" s="96"/>
       <c r="G43" s="97" t="str">
         <f>VLOOKUP(O3,_xlfn._TRO_TRAILING(T:V),3,0)</f>
-        <v>Ibrahim Akgün</v>
+        <v>Nurettin Biçer</v>
       </c>
       <c r="H43" s="98"/>
       <c r="I43" s="99"/>

</xml_diff>